<commit_message>
New Update with correction to the reference year- Poverty and deprivation not included
</commit_message>
<xml_diff>
--- a/data/health/Life expectancy inequalities in the South West/Life expectancy inequality at birth by local authority in the South West, 2022 - 24.xlsx
+++ b/data/health/Life expectancy inequalities in the South West/Life expectancy inequality at birth by local authority in the South West, 2022 - 24.xlsx
@@ -3577,7 +3577,7 @@
       <c r="AI2" s="2" t="inlineStr"/>
       <c r="AJ2" s="2" t="inlineStr">
         <is>
-          <t>2026-07-21</t>
+          <t>2026-07-22</t>
         </is>
       </c>
     </row>
@@ -3699,7 +3699,7 @@
       <c r="AI3" s="2" t="inlineStr"/>
       <c r="AJ3" s="2" t="inlineStr">
         <is>
-          <t>2026-07-21</t>
+          <t>2026-07-22</t>
         </is>
       </c>
     </row>
@@ -3825,7 +3825,7 @@
       <c r="AI4" s="2" t="inlineStr"/>
       <c r="AJ4" s="2" t="inlineStr">
         <is>
-          <t>2026-07-21</t>
+          <t>2026-07-22</t>
         </is>
       </c>
     </row>
@@ -3947,7 +3947,7 @@
       <c r="AI5" s="2" t="inlineStr"/>
       <c r="AJ5" s="2" t="inlineStr">
         <is>
-          <t>2026-07-21</t>
+          <t>2026-07-22</t>
         </is>
       </c>
     </row>
@@ -4073,7 +4073,7 @@
       <c r="AI6" s="2" t="inlineStr"/>
       <c r="AJ6" s="2" t="inlineStr">
         <is>
-          <t>2026-07-21</t>
+          <t>2026-07-22</t>
         </is>
       </c>
     </row>
@@ -4195,7 +4195,7 @@
       <c r="AI7" s="2" t="inlineStr"/>
       <c r="AJ7" s="2" t="inlineStr">
         <is>
-          <t>2026-07-21</t>
+          <t>2026-07-22</t>
         </is>
       </c>
     </row>
@@ -4321,7 +4321,7 @@
       <c r="AI8" s="2" t="inlineStr"/>
       <c r="AJ8" s="2" t="inlineStr">
         <is>
-          <t>2026-07-21</t>
+          <t>2026-07-22</t>
         </is>
       </c>
     </row>
@@ -4443,7 +4443,7 @@
       <c r="AI9" s="2" t="inlineStr"/>
       <c r="AJ9" s="2" t="inlineStr">
         <is>
-          <t>2026-07-21</t>
+          <t>2026-07-22</t>
         </is>
       </c>
     </row>
@@ -4569,7 +4569,7 @@
       <c r="AI10" s="2" t="inlineStr"/>
       <c r="AJ10" s="2" t="inlineStr">
         <is>
-          <t>2026-07-21</t>
+          <t>2026-07-22</t>
         </is>
       </c>
     </row>
@@ -4691,7 +4691,7 @@
       <c r="AI11" s="2" t="inlineStr"/>
       <c r="AJ11" s="2" t="inlineStr">
         <is>
-          <t>2026-07-21</t>
+          <t>2026-07-22</t>
         </is>
       </c>
     </row>
@@ -4817,7 +4817,7 @@
       <c r="AI12" s="2" t="inlineStr"/>
       <c r="AJ12" s="2" t="inlineStr">
         <is>
-          <t>2026-07-21</t>
+          <t>2026-07-22</t>
         </is>
       </c>
     </row>
@@ -4939,7 +4939,7 @@
       <c r="AI13" s="2" t="inlineStr"/>
       <c r="AJ13" s="2" t="inlineStr">
         <is>
-          <t>2026-07-21</t>
+          <t>2026-07-22</t>
         </is>
       </c>
     </row>
@@ -5065,7 +5065,7 @@
       <c r="AI14" s="2" t="inlineStr"/>
       <c r="AJ14" s="2" t="inlineStr">
         <is>
-          <t>2026-07-21</t>
+          <t>2026-07-22</t>
         </is>
       </c>
     </row>
@@ -5187,7 +5187,7 @@
       <c r="AI15" s="2" t="inlineStr"/>
       <c r="AJ15" s="2" t="inlineStr">
         <is>
-          <t>2026-07-21</t>
+          <t>2026-07-22</t>
         </is>
       </c>
     </row>
@@ -5313,7 +5313,7 @@
       <c r="AI16" s="2" t="inlineStr"/>
       <c r="AJ16" s="2" t="inlineStr">
         <is>
-          <t>2026-07-21</t>
+          <t>2026-07-22</t>
         </is>
       </c>
     </row>
@@ -5435,7 +5435,7 @@
       <c r="AI17" s="2" t="inlineStr"/>
       <c r="AJ17" s="2" t="inlineStr">
         <is>
-          <t>2026-07-21</t>
+          <t>2026-07-22</t>
         </is>
       </c>
     </row>
@@ -5561,7 +5561,7 @@
       <c r="AI18" s="2" t="inlineStr"/>
       <c r="AJ18" s="2" t="inlineStr">
         <is>
-          <t>2026-07-21</t>
+          <t>2026-07-22</t>
         </is>
       </c>
     </row>
@@ -5683,7 +5683,7 @@
       <c r="AI19" s="2" t="inlineStr"/>
       <c r="AJ19" s="2" t="inlineStr">
         <is>
-          <t>2026-07-21</t>
+          <t>2026-07-22</t>
         </is>
       </c>
     </row>
@@ -5809,7 +5809,7 @@
       <c r="AI20" s="2" t="inlineStr"/>
       <c r="AJ20" s="2" t="inlineStr">
         <is>
-          <t>2026-07-21</t>
+          <t>2026-07-22</t>
         </is>
       </c>
     </row>
@@ -5931,7 +5931,7 @@
       <c r="AI21" s="2" t="inlineStr"/>
       <c r="AJ21" s="2" t="inlineStr">
         <is>
-          <t>2026-07-21</t>
+          <t>2026-07-22</t>
         </is>
       </c>
     </row>
@@ -6057,7 +6057,7 @@
       <c r="AI22" s="2" t="inlineStr"/>
       <c r="AJ22" s="2" t="inlineStr">
         <is>
-          <t>2026-07-21</t>
+          <t>2026-07-22</t>
         </is>
       </c>
     </row>
@@ -6179,7 +6179,7 @@
       <c r="AI23" s="2" t="inlineStr"/>
       <c r="AJ23" s="2" t="inlineStr">
         <is>
-          <t>2026-07-21</t>
+          <t>2026-07-22</t>
         </is>
       </c>
     </row>
@@ -6305,7 +6305,7 @@
       <c r="AI24" s="2" t="inlineStr"/>
       <c r="AJ24" s="2" t="inlineStr">
         <is>
-          <t>2026-07-21</t>
+          <t>2026-07-22</t>
         </is>
       </c>
     </row>
@@ -6427,7 +6427,7 @@
       <c r="AI25" s="2" t="inlineStr"/>
       <c r="AJ25" s="2" t="inlineStr">
         <is>
-          <t>2026-07-21</t>
+          <t>2026-07-22</t>
         </is>
       </c>
     </row>
@@ -6553,7 +6553,7 @@
       <c r="AI26" s="2" t="inlineStr"/>
       <c r="AJ26" s="2" t="inlineStr">
         <is>
-          <t>2026-07-21</t>
+          <t>2026-07-22</t>
         </is>
       </c>
     </row>
@@ -6675,7 +6675,7 @@
       <c r="AI27" s="2" t="inlineStr"/>
       <c r="AJ27" s="2" t="inlineStr">
         <is>
-          <t>2026-07-21</t>
+          <t>2026-07-22</t>
         </is>
       </c>
     </row>
@@ -6801,7 +6801,7 @@
       <c r="AI28" s="2" t="inlineStr"/>
       <c r="AJ28" s="2" t="inlineStr">
         <is>
-          <t>2026-07-21</t>
+          <t>2026-07-22</t>
         </is>
       </c>
     </row>
@@ -6923,7 +6923,7 @@
       <c r="AI29" s="2" t="inlineStr"/>
       <c r="AJ29" s="2" t="inlineStr">
         <is>
-          <t>2026-07-21</t>
+          <t>2026-07-22</t>
         </is>
       </c>
     </row>
@@ -7049,7 +7049,7 @@
       <c r="AI30" s="2" t="inlineStr"/>
       <c r="AJ30" s="2" t="inlineStr">
         <is>
-          <t>2026-07-21</t>
+          <t>2026-07-22</t>
         </is>
       </c>
     </row>
@@ -7171,7 +7171,7 @@
       <c r="AI31" s="2" t="inlineStr"/>
       <c r="AJ31" s="2" t="inlineStr">
         <is>
-          <t>2026-07-21</t>
+          <t>2026-07-22</t>
         </is>
       </c>
     </row>
@@ -7297,7 +7297,7 @@
       <c r="AI32" s="2" t="inlineStr"/>
       <c r="AJ32" s="2" t="inlineStr">
         <is>
-          <t>2026-07-21</t>
+          <t>2026-07-22</t>
         </is>
       </c>
     </row>
@@ -7419,7 +7419,7 @@
       <c r="AI33" s="2" t="inlineStr"/>
       <c r="AJ33" s="2" t="inlineStr">
         <is>
-          <t>2026-07-21</t>
+          <t>2026-07-22</t>
         </is>
       </c>
     </row>
@@ -7545,7 +7545,7 @@
       <c r="AI34" s="2" t="inlineStr"/>
       <c r="AJ34" s="2" t="inlineStr">
         <is>
-          <t>2026-07-21</t>
+          <t>2026-07-22</t>
         </is>
       </c>
     </row>
@@ -7667,7 +7667,7 @@
       <c r="AI35" s="2" t="inlineStr"/>
       <c r="AJ35" s="2" t="inlineStr">
         <is>
-          <t>2026-07-21</t>
+          <t>2026-07-22</t>
         </is>
       </c>
     </row>
@@ -7793,7 +7793,7 @@
       <c r="AI36" s="2" t="inlineStr"/>
       <c r="AJ36" s="2" t="inlineStr">
         <is>
-          <t>2026-07-21</t>
+          <t>2026-07-22</t>
         </is>
       </c>
     </row>
@@ -7915,7 +7915,7 @@
       <c r="AI37" s="2" t="inlineStr"/>
       <c r="AJ37" s="2" t="inlineStr">
         <is>
-          <t>2026-07-21</t>
+          <t>2026-07-22</t>
         </is>
       </c>
     </row>
@@ -8041,7 +8041,7 @@
       <c r="AI38" s="2" t="inlineStr"/>
       <c r="AJ38" s="2" t="inlineStr">
         <is>
-          <t>2026-07-21</t>
+          <t>2026-07-22</t>
         </is>
       </c>
     </row>
@@ -8163,7 +8163,7 @@
       <c r="AI39" s="2" t="inlineStr"/>
       <c r="AJ39" s="2" t="inlineStr">
         <is>
-          <t>2026-07-21</t>
+          <t>2026-07-22</t>
         </is>
       </c>
     </row>
@@ -8289,7 +8289,7 @@
       <c r="AI40" s="2" t="inlineStr"/>
       <c r="AJ40" s="2" t="inlineStr">
         <is>
-          <t>2026-07-21</t>
+          <t>2026-07-22</t>
         </is>
       </c>
     </row>
@@ -8411,7 +8411,7 @@
       <c r="AI41" s="2" t="inlineStr"/>
       <c r="AJ41" s="2" t="inlineStr">
         <is>
-          <t>2026-07-21</t>
+          <t>2026-07-22</t>
         </is>
       </c>
     </row>
@@ -8537,7 +8537,7 @@
       </c>
       <c r="B9" s="6" t="inlineStr">
         <is>
-          <t>2026-07-21</t>
+          <t>2026-07-22</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
New update on health data - observation sheet
</commit_message>
<xml_diff>
--- a/data/health/Life expectancy inequalities in the South West/Life expectancy inequality at birth by local authority in the South West, 2022 - 24.xlsx
+++ b/data/health/Life expectancy inequalities in the South West/Life expectancy inequality at birth by local authority in the South West, 2022 - 24.xlsx
@@ -3232,7 +3232,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:AJ41"/>
+  <dimension ref="A1:AJ21"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="24" customWidth="1" min="1" max="1"/>
@@ -3265,7 +3265,7 @@
     <col width="17" customWidth="1" min="28" max="28"/>
     <col width="21" customWidth="1" min="29" max="29"/>
     <col width="30" customWidth="1" min="30" max="30"/>
-    <col width="36" customWidth="1" min="31" max="31"/>
+    <col width="20" customWidth="1" min="31" max="31"/>
     <col width="23" customWidth="1" min="32" max="32"/>
     <col width="20" customWidth="1" min="33" max="33"/>
     <col width="21" customWidth="1" min="34" max="34"/>
@@ -3651,7 +3651,7 @@
         </is>
       </c>
       <c r="O3" s="2" t="n">
-        <v>82.622937180088</v>
+        <v>7.9202826321953</v>
       </c>
       <c r="P3" s="2" t="inlineStr">
         <is>
@@ -3663,12 +3663,16 @@
       <c r="S3" s="2" t="inlineStr"/>
       <c r="T3" s="2" t="inlineStr"/>
       <c r="U3" s="2" t="inlineStr"/>
-      <c r="V3" s="2" t="n"/>
-      <c r="W3" s="2" t="n"/>
+      <c r="V3" s="2" t="n">
+        <v>6.26132478068758</v>
+      </c>
+      <c r="W3" s="2" t="n">
+        <v>9.579694105638771</v>
+      </c>
       <c r="X3" s="2" t="inlineStr"/>
       <c r="Y3" s="2" t="inlineStr">
         <is>
-          <t>Female</t>
+          <t>Male</t>
         </is>
       </c>
       <c r="Z3" s="2" t="inlineStr"/>
@@ -3676,7 +3680,7 @@
       <c r="AB3" s="2" t="inlineStr"/>
       <c r="AC3" s="2" t="inlineStr">
         <is>
-          <t>{"sex": "Female"}</t>
+          <t>{"sex": "Male"}</t>
         </is>
       </c>
       <c r="AD3" s="2" t="inlineStr">
@@ -3686,7 +3690,7 @@
       </c>
       <c r="AE3" s="2" t="inlineStr">
         <is>
-          <t>Limits for SII regression charts</t>
+          <t>SII value</t>
         </is>
       </c>
       <c r="AF3" s="2" t="inlineStr"/>
@@ -3739,22 +3743,22 @@
       </c>
       <c r="H4" s="2" t="inlineStr">
         <is>
-          <t>Bath and North East Somerset</t>
+          <t>Bristol, City of</t>
         </is>
       </c>
       <c r="I4" s="2" t="inlineStr">
         <is>
-          <t>E06000022</t>
+          <t>E06000023</t>
         </is>
       </c>
       <c r="J4" s="2" t="inlineStr">
         <is>
-          <t>Bath and North East Somerset</t>
+          <t>Bristol, City of</t>
         </is>
       </c>
       <c r="K4" s="2" t="inlineStr">
         <is>
-          <t>E06000022</t>
+          <t>E06000023</t>
         </is>
       </c>
       <c r="L4" s="2" t="inlineStr">
@@ -3773,7 +3777,7 @@
         </is>
       </c>
       <c r="O4" s="2" t="n">
-        <v>7.9202826321953</v>
+        <v>7.30452963126084</v>
       </c>
       <c r="P4" s="2" t="inlineStr">
         <is>
@@ -3786,15 +3790,15 @@
       <c r="T4" s="2" t="inlineStr"/>
       <c r="U4" s="2" t="inlineStr"/>
       <c r="V4" s="2" t="n">
-        <v>6.26132478068758</v>
+        <v>6.20913134168222</v>
       </c>
       <c r="W4" s="2" t="n">
-        <v>9.579694105638771</v>
+        <v>8.39874238602116</v>
       </c>
       <c r="X4" s="2" t="inlineStr"/>
       <c r="Y4" s="2" t="inlineStr">
         <is>
-          <t>Male</t>
+          <t>Female</t>
         </is>
       </c>
       <c r="Z4" s="2" t="inlineStr"/>
@@ -3802,7 +3806,7 @@
       <c r="AB4" s="2" t="inlineStr"/>
       <c r="AC4" s="2" t="inlineStr">
         <is>
-          <t>{"sex": "Male"}</t>
+          <t>{"sex": "Female"}</t>
         </is>
       </c>
       <c r="AD4" s="2" t="inlineStr">
@@ -3865,22 +3869,22 @@
       </c>
       <c r="H5" s="2" t="inlineStr">
         <is>
-          <t>Bath and North East Somerset</t>
+          <t>Bristol, City of</t>
         </is>
       </c>
       <c r="I5" s="2" t="inlineStr">
         <is>
-          <t>E06000022</t>
+          <t>E06000023</t>
         </is>
       </c>
       <c r="J5" s="2" t="inlineStr">
         <is>
-          <t>Bath and North East Somerset</t>
+          <t>Bristol, City of</t>
         </is>
       </c>
       <c r="K5" s="2" t="inlineStr">
         <is>
-          <t>E06000022</t>
+          <t>E06000023</t>
         </is>
       </c>
       <c r="L5" s="2" t="inlineStr">
@@ -3899,7 +3903,7 @@
         </is>
       </c>
       <c r="O5" s="2" t="n">
-        <v>77.4420584193702</v>
+        <v>10.5429500425896</v>
       </c>
       <c r="P5" s="2" t="inlineStr">
         <is>
@@ -3911,8 +3915,12 @@
       <c r="S5" s="2" t="inlineStr"/>
       <c r="T5" s="2" t="inlineStr"/>
       <c r="U5" s="2" t="inlineStr"/>
-      <c r="V5" s="2" t="n"/>
-      <c r="W5" s="2" t="n"/>
+      <c r="V5" s="2" t="n">
+        <v>9.433027688260321</v>
+      </c>
+      <c r="W5" s="2" t="n">
+        <v>11.6533063685318</v>
+      </c>
       <c r="X5" s="2" t="inlineStr"/>
       <c r="Y5" s="2" t="inlineStr">
         <is>
@@ -3934,7 +3942,7 @@
       </c>
       <c r="AE5" s="2" t="inlineStr">
         <is>
-          <t>Limits for SII regression charts</t>
+          <t>SII value</t>
         </is>
       </c>
       <c r="AF5" s="2" t="inlineStr"/>
@@ -3987,22 +3995,22 @@
       </c>
       <c r="H6" s="2" t="inlineStr">
         <is>
-          <t>Bristol, City of</t>
+          <t>Gloucestershire</t>
         </is>
       </c>
       <c r="I6" s="2" t="inlineStr">
         <is>
-          <t>E06000023</t>
+          <t>E10000013</t>
         </is>
       </c>
       <c r="J6" s="2" t="inlineStr">
         <is>
-          <t>Bristol, City of</t>
+          <t>Gloucestershire</t>
         </is>
       </c>
       <c r="K6" s="2" t="inlineStr">
         <is>
-          <t>E06000023</t>
+          <t>E10000013</t>
         </is>
       </c>
       <c r="L6" s="2" t="inlineStr">
@@ -4021,7 +4029,7 @@
         </is>
       </c>
       <c r="O6" s="2" t="n">
-        <v>7.30452963126084</v>
+        <v>6.34854202991486</v>
       </c>
       <c r="P6" s="2" t="inlineStr">
         <is>
@@ -4034,10 +4042,10 @@
       <c r="T6" s="2" t="inlineStr"/>
       <c r="U6" s="2" t="inlineStr"/>
       <c r="V6" s="2" t="n">
-        <v>6.20913134168222</v>
+        <v>5.52619634239314</v>
       </c>
       <c r="W6" s="2" t="n">
-        <v>8.39874238602116</v>
+        <v>7.16841812129896</v>
       </c>
       <c r="X6" s="2" t="inlineStr"/>
       <c r="Y6" s="2" t="inlineStr">
@@ -4113,22 +4121,22 @@
       </c>
       <c r="H7" s="2" t="inlineStr">
         <is>
-          <t>Bristol, City of</t>
+          <t>Gloucestershire</t>
         </is>
       </c>
       <c r="I7" s="2" t="inlineStr">
         <is>
-          <t>E06000023</t>
+          <t>E10000013</t>
         </is>
       </c>
       <c r="J7" s="2" t="inlineStr">
         <is>
-          <t>Bristol, City of</t>
+          <t>Gloucestershire</t>
         </is>
       </c>
       <c r="K7" s="2" t="inlineStr">
         <is>
-          <t>E06000023</t>
+          <t>E10000013</t>
         </is>
       </c>
       <c r="L7" s="2" t="inlineStr">
@@ -4147,7 +4155,7 @@
         </is>
       </c>
       <c r="O7" s="2" t="n">
-        <v>79.35731424745531</v>
+        <v>8.06754586264559</v>
       </c>
       <c r="P7" s="2" t="inlineStr">
         <is>
@@ -4159,12 +4167,16 @@
       <c r="S7" s="2" t="inlineStr"/>
       <c r="T7" s="2" t="inlineStr"/>
       <c r="U7" s="2" t="inlineStr"/>
-      <c r="V7" s="2" t="n"/>
-      <c r="W7" s="2" t="n"/>
+      <c r="V7" s="2" t="n">
+        <v>7.17112499799161</v>
+      </c>
+      <c r="W7" s="2" t="n">
+        <v>8.96359406622302</v>
+      </c>
       <c r="X7" s="2" t="inlineStr"/>
       <c r="Y7" s="2" t="inlineStr">
         <is>
-          <t>Female</t>
+          <t>Male</t>
         </is>
       </c>
       <c r="Z7" s="2" t="inlineStr"/>
@@ -4172,7 +4184,7 @@
       <c r="AB7" s="2" t="inlineStr"/>
       <c r="AC7" s="2" t="inlineStr">
         <is>
-          <t>{"sex": "Female"}</t>
+          <t>{"sex": "Male"}</t>
         </is>
       </c>
       <c r="AD7" s="2" t="inlineStr">
@@ -4182,7 +4194,7 @@
       </c>
       <c r="AE7" s="2" t="inlineStr">
         <is>
-          <t>Limits for SII regression charts</t>
+          <t>SII value</t>
         </is>
       </c>
       <c r="AF7" s="2" t="inlineStr"/>
@@ -4235,22 +4247,22 @@
       </c>
       <c r="H8" s="2" t="inlineStr">
         <is>
-          <t>Bristol, City of</t>
+          <t>North Somerset</t>
         </is>
       </c>
       <c r="I8" s="2" t="inlineStr">
         <is>
-          <t>E06000023</t>
+          <t>E06000024</t>
         </is>
       </c>
       <c r="J8" s="2" t="inlineStr">
         <is>
-          <t>Bristol, City of</t>
+          <t>North Somerset</t>
         </is>
       </c>
       <c r="K8" s="2" t="inlineStr">
         <is>
-          <t>E06000023</t>
+          <t>E06000024</t>
         </is>
       </c>
       <c r="L8" s="2" t="inlineStr">
@@ -4269,7 +4281,7 @@
         </is>
       </c>
       <c r="O8" s="2" t="n">
-        <v>10.5429500425896</v>
+        <v>7.4999326415297</v>
       </c>
       <c r="P8" s="2" t="inlineStr">
         <is>
@@ -4282,15 +4294,15 @@
       <c r="T8" s="2" t="inlineStr"/>
       <c r="U8" s="2" t="inlineStr"/>
       <c r="V8" s="2" t="n">
-        <v>9.433027688260321</v>
+        <v>6.14154897644448</v>
       </c>
       <c r="W8" s="2" t="n">
-        <v>11.6533063685318</v>
+        <v>8.85926735146522</v>
       </c>
       <c r="X8" s="2" t="inlineStr"/>
       <c r="Y8" s="2" t="inlineStr">
         <is>
-          <t>Male</t>
+          <t>Female</t>
         </is>
       </c>
       <c r="Z8" s="2" t="inlineStr"/>
@@ -4298,7 +4310,7 @@
       <c r="AB8" s="2" t="inlineStr"/>
       <c r="AC8" s="2" t="inlineStr">
         <is>
-          <t>{"sex": "Male"}</t>
+          <t>{"sex": "Female"}</t>
         </is>
       </c>
       <c r="AD8" s="2" t="inlineStr">
@@ -4361,22 +4373,22 @@
       </c>
       <c r="H9" s="2" t="inlineStr">
         <is>
-          <t>Bristol, City of</t>
+          <t>North Somerset</t>
         </is>
       </c>
       <c r="I9" s="2" t="inlineStr">
         <is>
-          <t>E06000023</t>
+          <t>E06000024</t>
         </is>
       </c>
       <c r="J9" s="2" t="inlineStr">
         <is>
-          <t>Bristol, City of</t>
+          <t>North Somerset</t>
         </is>
       </c>
       <c r="K9" s="2" t="inlineStr">
         <is>
-          <t>E06000023</t>
+          <t>E06000024</t>
         </is>
       </c>
       <c r="L9" s="2" t="inlineStr">
@@ -4395,7 +4407,7 @@
         </is>
       </c>
       <c r="O9" s="2" t="n">
-        <v>73.3476633344378</v>
+        <v>9.156046355609829</v>
       </c>
       <c r="P9" s="2" t="inlineStr">
         <is>
@@ -4407,8 +4419,12 @@
       <c r="S9" s="2" t="inlineStr"/>
       <c r="T9" s="2" t="inlineStr"/>
       <c r="U9" s="2" t="inlineStr"/>
-      <c r="V9" s="2" t="n"/>
-      <c r="W9" s="2" t="n"/>
+      <c r="V9" s="2" t="n">
+        <v>7.59661443050507</v>
+      </c>
+      <c r="W9" s="2" t="n">
+        <v>10.7145021296448</v>
+      </c>
       <c r="X9" s="2" t="inlineStr"/>
       <c r="Y9" s="2" t="inlineStr">
         <is>
@@ -4430,7 +4446,7 @@
       </c>
       <c r="AE9" s="2" t="inlineStr">
         <is>
-          <t>Limits for SII regression charts</t>
+          <t>SII value</t>
         </is>
       </c>
       <c r="AF9" s="2" t="inlineStr"/>
@@ -4483,22 +4499,22 @@
       </c>
       <c r="H10" s="2" t="inlineStr">
         <is>
-          <t>Gloucestershire</t>
+          <t>South Gloucestershire</t>
         </is>
       </c>
       <c r="I10" s="2" t="inlineStr">
         <is>
-          <t>E10000013</t>
+          <t>E06000025</t>
         </is>
       </c>
       <c r="J10" s="2" t="inlineStr">
         <is>
-          <t>Gloucestershire</t>
+          <t>South Gloucestershire</t>
         </is>
       </c>
       <c r="K10" s="2" t="inlineStr">
         <is>
-          <t>E10000013</t>
+          <t>E06000025</t>
         </is>
       </c>
       <c r="L10" s="2" t="inlineStr">
@@ -4517,7 +4533,7 @@
         </is>
       </c>
       <c r="O10" s="2" t="n">
-        <v>6.34854202991486</v>
+        <v>6.40771973321451</v>
       </c>
       <c r="P10" s="2" t="inlineStr">
         <is>
@@ -4530,10 +4546,10 @@
       <c r="T10" s="2" t="inlineStr"/>
       <c r="U10" s="2" t="inlineStr"/>
       <c r="V10" s="2" t="n">
-        <v>5.52619634239314</v>
+        <v>4.97826164111792</v>
       </c>
       <c r="W10" s="2" t="n">
-        <v>7.16841812129896</v>
+        <v>7.84397740405498</v>
       </c>
       <c r="X10" s="2" t="inlineStr"/>
       <c r="Y10" s="2" t="inlineStr">
@@ -4609,22 +4625,22 @@
       </c>
       <c r="H11" s="2" t="inlineStr">
         <is>
-          <t>Gloucestershire</t>
+          <t>South Gloucestershire</t>
         </is>
       </c>
       <c r="I11" s="2" t="inlineStr">
         <is>
-          <t>E10000013</t>
+          <t>E06000025</t>
         </is>
       </c>
       <c r="J11" s="2" t="inlineStr">
         <is>
-          <t>Gloucestershire</t>
+          <t>South Gloucestershire</t>
         </is>
       </c>
       <c r="K11" s="2" t="inlineStr">
         <is>
-          <t>E10000013</t>
+          <t>E06000025</t>
         </is>
       </c>
       <c r="L11" s="2" t="inlineStr">
@@ -4643,7 +4659,7 @@
         </is>
       </c>
       <c r="O11" s="2" t="n">
-        <v>80.6996015823586</v>
+        <v>6.77044528853804</v>
       </c>
       <c r="P11" s="2" t="inlineStr">
         <is>
@@ -4655,12 +4671,16 @@
       <c r="S11" s="2" t="inlineStr"/>
       <c r="T11" s="2" t="inlineStr"/>
       <c r="U11" s="2" t="inlineStr"/>
-      <c r="V11" s="2" t="n"/>
-      <c r="W11" s="2" t="n"/>
+      <c r="V11" s="2" t="n">
+        <v>5.51532525439773</v>
+      </c>
+      <c r="W11" s="2" t="n">
+        <v>8.02653045374093</v>
+      </c>
       <c r="X11" s="2" t="inlineStr"/>
       <c r="Y11" s="2" t="inlineStr">
         <is>
-          <t>Female</t>
+          <t>Male</t>
         </is>
       </c>
       <c r="Z11" s="2" t="inlineStr"/>
@@ -4668,7 +4688,7 @@
       <c r="AB11" s="2" t="inlineStr"/>
       <c r="AC11" s="2" t="inlineStr">
         <is>
-          <t>{"sex": "Female"}</t>
+          <t>{"sex": "Male"}</t>
         </is>
       </c>
       <c r="AD11" s="2" t="inlineStr">
@@ -4678,7 +4698,7 @@
       </c>
       <c r="AE11" s="2" t="inlineStr">
         <is>
-          <t>Limits for SII regression charts</t>
+          <t>SII value</t>
         </is>
       </c>
       <c r="AF11" s="2" t="inlineStr"/>
@@ -4731,22 +4751,22 @@
       </c>
       <c r="H12" s="2" t="inlineStr">
         <is>
-          <t>Gloucestershire</t>
+          <t>Swindon</t>
         </is>
       </c>
       <c r="I12" s="2" t="inlineStr">
         <is>
-          <t>E10000013</t>
+          <t>E06000030</t>
         </is>
       </c>
       <c r="J12" s="2" t="inlineStr">
         <is>
-          <t>Gloucestershire</t>
+          <t>Swindon</t>
         </is>
       </c>
       <c r="K12" s="2" t="inlineStr">
         <is>
-          <t>E10000013</t>
+          <t>E06000030</t>
         </is>
       </c>
       <c r="L12" s="2" t="inlineStr">
@@ -4765,7 +4785,7 @@
         </is>
       </c>
       <c r="O12" s="2" t="n">
-        <v>8.06754586264559</v>
+        <v>5.67937352872535</v>
       </c>
       <c r="P12" s="2" t="inlineStr">
         <is>
@@ -4778,15 +4798,15 @@
       <c r="T12" s="2" t="inlineStr"/>
       <c r="U12" s="2" t="inlineStr"/>
       <c r="V12" s="2" t="n">
-        <v>7.17112499799161</v>
+        <v>4.23304060137117</v>
       </c>
       <c r="W12" s="2" t="n">
-        <v>8.96359406622302</v>
+        <v>7.12145672576508</v>
       </c>
       <c r="X12" s="2" t="inlineStr"/>
       <c r="Y12" s="2" t="inlineStr">
         <is>
-          <t>Male</t>
+          <t>Female</t>
         </is>
       </c>
       <c r="Z12" s="2" t="inlineStr"/>
@@ -4794,7 +4814,7 @@
       <c r="AB12" s="2" t="inlineStr"/>
       <c r="AC12" s="2" t="inlineStr">
         <is>
-          <t>{"sex": "Male"}</t>
+          <t>{"sex": "Female"}</t>
         </is>
       </c>
       <c r="AD12" s="2" t="inlineStr">
@@ -4857,22 +4877,22 @@
       </c>
       <c r="H13" s="2" t="inlineStr">
         <is>
-          <t>Gloucestershire</t>
+          <t>Swindon</t>
         </is>
       </c>
       <c r="I13" s="2" t="inlineStr">
         <is>
-          <t>E10000013</t>
+          <t>E06000030</t>
         </is>
       </c>
       <c r="J13" s="2" t="inlineStr">
         <is>
-          <t>Gloucestershire</t>
+          <t>Swindon</t>
         </is>
       </c>
       <c r="K13" s="2" t="inlineStr">
         <is>
-          <t>E10000013</t>
+          <t>E06000030</t>
         </is>
       </c>
       <c r="L13" s="2" t="inlineStr">
@@ -4891,7 +4911,7 @@
         </is>
       </c>
       <c r="O13" s="2" t="n">
-        <v>76.2345935933421</v>
+        <v>9.97135672505077</v>
       </c>
       <c r="P13" s="2" t="inlineStr">
         <is>
@@ -4903,8 +4923,12 @@
       <c r="S13" s="2" t="inlineStr"/>
       <c r="T13" s="2" t="inlineStr"/>
       <c r="U13" s="2" t="inlineStr"/>
-      <c r="V13" s="2" t="n"/>
-      <c r="W13" s="2" t="n"/>
+      <c r="V13" s="2" t="n">
+        <v>8.47354893144897</v>
+      </c>
+      <c r="W13" s="2" t="n">
+        <v>11.4659628814125</v>
+      </c>
       <c r="X13" s="2" t="inlineStr"/>
       <c r="Y13" s="2" t="inlineStr">
         <is>
@@ -4926,7 +4950,7 @@
       </c>
       <c r="AE13" s="2" t="inlineStr">
         <is>
-          <t>Limits for SII regression charts</t>
+          <t>SII value</t>
         </is>
       </c>
       <c r="AF13" s="2" t="inlineStr"/>
@@ -4979,22 +5003,22 @@
       </c>
       <c r="H14" s="2" t="inlineStr">
         <is>
-          <t>North Somerset</t>
+          <t>Wiltshire</t>
         </is>
       </c>
       <c r="I14" s="2" t="inlineStr">
         <is>
-          <t>E06000024</t>
+          <t>E06000054</t>
         </is>
       </c>
       <c r="J14" s="2" t="inlineStr">
         <is>
-          <t>North Somerset</t>
+          <t>Wiltshire</t>
         </is>
       </c>
       <c r="K14" s="2" t="inlineStr">
         <is>
-          <t>E06000024</t>
+          <t>E06000054</t>
         </is>
       </c>
       <c r="L14" s="2" t="inlineStr">
@@ -5013,7 +5037,7 @@
         </is>
       </c>
       <c r="O14" s="2" t="n">
-        <v>7.4999326415297</v>
+        <v>3.68786604792967</v>
       </c>
       <c r="P14" s="2" t="inlineStr">
         <is>
@@ -5026,10 +5050,10 @@
       <c r="T14" s="2" t="inlineStr"/>
       <c r="U14" s="2" t="inlineStr"/>
       <c r="V14" s="2" t="n">
-        <v>6.14154897644448</v>
+        <v>2.74496766069945</v>
       </c>
       <c r="W14" s="2" t="n">
-        <v>8.85926735146522</v>
+        <v>4.62779265274191</v>
       </c>
       <c r="X14" s="2" t="inlineStr"/>
       <c r="Y14" s="2" t="inlineStr">
@@ -5105,22 +5129,22 @@
       </c>
       <c r="H15" s="2" t="inlineStr">
         <is>
-          <t>North Somerset</t>
+          <t>Wiltshire</t>
         </is>
       </c>
       <c r="I15" s="2" t="inlineStr">
         <is>
-          <t>E06000024</t>
+          <t>E06000054</t>
         </is>
       </c>
       <c r="J15" s="2" t="inlineStr">
         <is>
-          <t>North Somerset</t>
+          <t>Wiltshire</t>
         </is>
       </c>
       <c r="K15" s="2" t="inlineStr">
         <is>
-          <t>E06000024</t>
+          <t>E06000054</t>
         </is>
       </c>
       <c r="L15" s="2" t="inlineStr">
@@ -5139,7 +5163,7 @@
         </is>
       </c>
       <c r="O15" s="2" t="n">
-        <v>80.59901757353281</v>
+        <v>4.91994895362696</v>
       </c>
       <c r="P15" s="2" t="inlineStr">
         <is>
@@ -5151,12 +5175,16 @@
       <c r="S15" s="2" t="inlineStr"/>
       <c r="T15" s="2" t="inlineStr"/>
       <c r="U15" s="2" t="inlineStr"/>
-      <c r="V15" s="2" t="n"/>
-      <c r="W15" s="2" t="n"/>
+      <c r="V15" s="2" t="n">
+        <v>3.92504759854335</v>
+      </c>
+      <c r="W15" s="2" t="n">
+        <v>5.91316284510629</v>
+      </c>
       <c r="X15" s="2" t="inlineStr"/>
       <c r="Y15" s="2" t="inlineStr">
         <is>
-          <t>Female</t>
+          <t>Male</t>
         </is>
       </c>
       <c r="Z15" s="2" t="inlineStr"/>
@@ -5164,7 +5192,7 @@
       <c r="AB15" s="2" t="inlineStr"/>
       <c r="AC15" s="2" t="inlineStr">
         <is>
-          <t>{"sex": "Female"}</t>
+          <t>{"sex": "Male"}</t>
         </is>
       </c>
       <c r="AD15" s="2" t="inlineStr">
@@ -5174,7 +5202,7 @@
       </c>
       <c r="AE15" s="2" t="inlineStr">
         <is>
-          <t>Limits for SII regression charts</t>
+          <t>SII value</t>
         </is>
       </c>
       <c r="AF15" s="2" t="inlineStr"/>
@@ -5227,27 +5255,27 @@
       </c>
       <c r="H16" s="2" t="inlineStr">
         <is>
-          <t>North Somerset</t>
+          <t>England</t>
         </is>
       </c>
       <c r="I16" s="2" t="inlineStr">
         <is>
-          <t>E06000024</t>
+          <t>E92000001</t>
         </is>
       </c>
       <c r="J16" s="2" t="inlineStr">
         <is>
-          <t>North Somerset</t>
+          <t>England</t>
         </is>
       </c>
       <c r="K16" s="2" t="inlineStr">
         <is>
-          <t>E06000024</t>
+          <t>E92000001</t>
         </is>
       </c>
       <c r="L16" s="2" t="inlineStr">
         <is>
-          <t>local_authority</t>
+          <t>country</t>
         </is>
       </c>
       <c r="M16" s="2" t="inlineStr">
@@ -5261,7 +5289,7 @@
         </is>
       </c>
       <c r="O16" s="2" t="n">
-        <v>9.156046355609829</v>
+        <v>8.029185211892139</v>
       </c>
       <c r="P16" s="2" t="inlineStr">
         <is>
@@ -5274,15 +5302,15 @@
       <c r="T16" s="2" t="inlineStr"/>
       <c r="U16" s="2" t="inlineStr"/>
       <c r="V16" s="2" t="n">
-        <v>7.59661443050507</v>
+        <v>7.9351805783358</v>
       </c>
       <c r="W16" s="2" t="n">
-        <v>10.7145021296448</v>
+        <v>8.12327840388291</v>
       </c>
       <c r="X16" s="2" t="inlineStr"/>
       <c r="Y16" s="2" t="inlineStr">
         <is>
-          <t>Male</t>
+          <t>Female</t>
         </is>
       </c>
       <c r="Z16" s="2" t="inlineStr"/>
@@ -5290,7 +5318,7 @@
       <c r="AB16" s="2" t="inlineStr"/>
       <c r="AC16" s="2" t="inlineStr">
         <is>
-          <t>{"sex": "Male"}</t>
+          <t>{"sex": "Female"}</t>
         </is>
       </c>
       <c r="AD16" s="2" t="inlineStr">
@@ -5353,27 +5381,27 @@
       </c>
       <c r="H17" s="2" t="inlineStr">
         <is>
-          <t>North Somerset</t>
+          <t>England</t>
         </is>
       </c>
       <c r="I17" s="2" t="inlineStr">
         <is>
-          <t>E06000024</t>
+          <t>E92000001</t>
         </is>
       </c>
       <c r="J17" s="2" t="inlineStr">
         <is>
-          <t>North Somerset</t>
+          <t>England</t>
         </is>
       </c>
       <c r="K17" s="2" t="inlineStr">
         <is>
-          <t>E06000024</t>
+          <t>E92000001</t>
         </is>
       </c>
       <c r="L17" s="2" t="inlineStr">
         <is>
-          <t>local_authority</t>
+          <t>country</t>
         </is>
       </c>
       <c r="M17" s="2" t="inlineStr">
@@ -5387,7 +5415,7 @@
         </is>
       </c>
       <c r="O17" s="2" t="n">
-        <v>76.36393130106789</v>
+        <v>10.373953779621</v>
       </c>
       <c r="P17" s="2" t="inlineStr">
         <is>
@@ -5399,8 +5427,12 @@
       <c r="S17" s="2" t="inlineStr"/>
       <c r="T17" s="2" t="inlineStr"/>
       <c r="U17" s="2" t="inlineStr"/>
-      <c r="V17" s="2" t="n"/>
-      <c r="W17" s="2" t="n"/>
+      <c r="V17" s="2" t="n">
+        <v>10.2754490660122</v>
+      </c>
+      <c r="W17" s="2" t="n">
+        <v>10.4724763027866</v>
+      </c>
       <c r="X17" s="2" t="inlineStr"/>
       <c r="Y17" s="2" t="inlineStr">
         <is>
@@ -5422,7 +5454,7 @@
       </c>
       <c r="AE17" s="2" t="inlineStr">
         <is>
-          <t>Limits for SII regression charts</t>
+          <t>SII value</t>
         </is>
       </c>
       <c r="AF17" s="2" t="inlineStr"/>
@@ -5475,27 +5507,27 @@
       </c>
       <c r="H18" s="2" t="inlineStr">
         <is>
-          <t>South Gloucestershire</t>
+          <t>South West region (statistical)</t>
         </is>
       </c>
       <c r="I18" s="2" t="inlineStr">
         <is>
-          <t>E06000025</t>
+          <t>E12000009</t>
         </is>
       </c>
       <c r="J18" s="2" t="inlineStr">
         <is>
-          <t>South Gloucestershire</t>
+          <t>South West region (statistical)</t>
         </is>
       </c>
       <c r="K18" s="2" t="inlineStr">
         <is>
-          <t>E06000025</t>
+          <t>E12000009</t>
         </is>
       </c>
       <c r="L18" s="2" t="inlineStr">
         <is>
-          <t>local_authority</t>
+          <t>region</t>
         </is>
       </c>
       <c r="M18" s="2" t="inlineStr">
@@ -5509,7 +5541,7 @@
         </is>
       </c>
       <c r="O18" s="2" t="n">
-        <v>6.40771973321451</v>
+        <v>5.59964175909663</v>
       </c>
       <c r="P18" s="2" t="inlineStr">
         <is>
@@ -5522,10 +5554,10 @@
       <c r="T18" s="2" t="inlineStr"/>
       <c r="U18" s="2" t="inlineStr"/>
       <c r="V18" s="2" t="n">
-        <v>4.97826164111792</v>
+        <v>5.31888872864678</v>
       </c>
       <c r="W18" s="2" t="n">
-        <v>7.84397740405498</v>
+        <v>5.88052225585969</v>
       </c>
       <c r="X18" s="2" t="inlineStr"/>
       <c r="Y18" s="2" t="inlineStr">
@@ -5601,27 +5633,27 @@
       </c>
       <c r="H19" s="2" t="inlineStr">
         <is>
-          <t>South Gloucestershire</t>
+          <t>South West region (statistical)</t>
         </is>
       </c>
       <c r="I19" s="2" t="inlineStr">
         <is>
-          <t>E06000025</t>
+          <t>E12000009</t>
         </is>
       </c>
       <c r="J19" s="2" t="inlineStr">
         <is>
-          <t>South Gloucestershire</t>
+          <t>South West region (statistical)</t>
         </is>
       </c>
       <c r="K19" s="2" t="inlineStr">
         <is>
-          <t>E06000025</t>
+          <t>E12000009</t>
         </is>
       </c>
       <c r="L19" s="2" t="inlineStr">
         <is>
-          <t>local_authority</t>
+          <t>region</t>
         </is>
       </c>
       <c r="M19" s="2" t="inlineStr">
@@ -5635,7 +5667,7 @@
         </is>
       </c>
       <c r="O19" s="2" t="n">
-        <v>81.58233605183661</v>
+        <v>7.78126329187077</v>
       </c>
       <c r="P19" s="2" t="inlineStr">
         <is>
@@ -5647,12 +5679,16 @@
       <c r="S19" s="2" t="inlineStr"/>
       <c r="T19" s="2" t="inlineStr"/>
       <c r="U19" s="2" t="inlineStr"/>
-      <c r="V19" s="2" t="n"/>
-      <c r="W19" s="2" t="n"/>
+      <c r="V19" s="2" t="n">
+        <v>7.4785922356622</v>
+      </c>
+      <c r="W19" s="2" t="n">
+        <v>8.08262609624769</v>
+      </c>
       <c r="X19" s="2" t="inlineStr"/>
       <c r="Y19" s="2" t="inlineStr">
         <is>
-          <t>Female</t>
+          <t>Male</t>
         </is>
       </c>
       <c r="Z19" s="2" t="inlineStr"/>
@@ -5660,7 +5696,7 @@
       <c r="AB19" s="2" t="inlineStr"/>
       <c r="AC19" s="2" t="inlineStr">
         <is>
-          <t>{"sex": "Female"}</t>
+          <t>{"sex": "Male"}</t>
         </is>
       </c>
       <c r="AD19" s="2" t="inlineStr">
@@ -5670,7 +5706,7 @@
       </c>
       <c r="AE19" s="2" t="inlineStr">
         <is>
-          <t>Limits for SII regression charts</t>
+          <t>SII value</t>
         </is>
       </c>
       <c r="AF19" s="2" t="inlineStr"/>
@@ -5723,27 +5759,27 @@
       </c>
       <c r="H20" s="2" t="inlineStr">
         <is>
-          <t>South Gloucestershire</t>
+          <t>London region (statistical)</t>
         </is>
       </c>
       <c r="I20" s="2" t="inlineStr">
         <is>
-          <t>E06000025</t>
+          <t>E12000007</t>
         </is>
       </c>
       <c r="J20" s="2" t="inlineStr">
         <is>
-          <t>South Gloucestershire</t>
+          <t>London region (statistical)</t>
         </is>
       </c>
       <c r="K20" s="2" t="inlineStr">
         <is>
-          <t>E06000025</t>
+          <t>E12000007</t>
         </is>
       </c>
       <c r="L20" s="2" t="inlineStr">
         <is>
-          <t>local_authority</t>
+          <t>region</t>
         </is>
       </c>
       <c r="M20" s="2" t="inlineStr">
@@ -5757,7 +5793,7 @@
         </is>
       </c>
       <c r="O20" s="2" t="n">
-        <v>6.77044528853804</v>
+        <v>4.74617067288794</v>
       </c>
       <c r="P20" s="2" t="inlineStr">
         <is>
@@ -5770,15 +5806,15 @@
       <c r="T20" s="2" t="inlineStr"/>
       <c r="U20" s="2" t="inlineStr"/>
       <c r="V20" s="2" t="n">
-        <v>5.51532525439773</v>
+        <v>4.4817708429787</v>
       </c>
       <c r="W20" s="2" t="n">
-        <v>8.02653045374093</v>
+        <v>5.00970035756127</v>
       </c>
       <c r="X20" s="2" t="inlineStr"/>
       <c r="Y20" s="2" t="inlineStr">
         <is>
-          <t>Male</t>
+          <t>Female</t>
         </is>
       </c>
       <c r="Z20" s="2" t="inlineStr"/>
@@ -5786,7 +5822,7 @@
       <c r="AB20" s="2" t="inlineStr"/>
       <c r="AC20" s="2" t="inlineStr">
         <is>
-          <t>{"sex": "Male"}</t>
+          <t>{"sex": "Female"}</t>
         </is>
       </c>
       <c r="AD20" s="2" t="inlineStr">
@@ -5849,27 +5885,27 @@
       </c>
       <c r="H21" s="2" t="inlineStr">
         <is>
-          <t>South Gloucestershire</t>
+          <t>London region (statistical)</t>
         </is>
       </c>
       <c r="I21" s="2" t="inlineStr">
         <is>
-          <t>E06000025</t>
+          <t>E12000007</t>
         </is>
       </c>
       <c r="J21" s="2" t="inlineStr">
         <is>
-          <t>South Gloucestershire</t>
+          <t>London region (statistical)</t>
         </is>
       </c>
       <c r="K21" s="2" t="inlineStr">
         <is>
-          <t>E06000025</t>
+          <t>E12000007</t>
         </is>
       </c>
       <c r="L21" s="2" t="inlineStr">
         <is>
-          <t>local_authority</t>
+          <t>region</t>
         </is>
       </c>
       <c r="M21" s="2" t="inlineStr">
@@ -5883,7 +5919,7 @@
         </is>
       </c>
       <c r="O21" s="2" t="n">
-        <v>77.6175520979706</v>
+        <v>7.85755327065507</v>
       </c>
       <c r="P21" s="2" t="inlineStr">
         <is>
@@ -5895,8 +5931,12 @@
       <c r="S21" s="2" t="inlineStr"/>
       <c r="T21" s="2" t="inlineStr"/>
       <c r="U21" s="2" t="inlineStr"/>
-      <c r="V21" s="2" t="n"/>
-      <c r="W21" s="2" t="n"/>
+      <c r="V21" s="2" t="n">
+        <v>7.58923901627381</v>
+      </c>
+      <c r="W21" s="2" t="n">
+        <v>8.125845973842219</v>
+      </c>
       <c r="X21" s="2" t="inlineStr"/>
       <c r="Y21" s="2" t="inlineStr">
         <is>
@@ -5918,7 +5958,7 @@
       </c>
       <c r="AE21" s="2" t="inlineStr">
         <is>
-          <t>Limits for SII regression charts</t>
+          <t>SII value</t>
         </is>
       </c>
       <c r="AF21" s="2" t="inlineStr"/>
@@ -5930,2486 +5970,6 @@
       <c r="AH21" s="2" t="inlineStr"/>
       <c r="AI21" s="2" t="inlineStr"/>
       <c r="AJ21" s="2" t="inlineStr">
-        <is>
-          <t>2026-07-22</t>
-        </is>
-      </c>
-    </row>
-    <row r="22">
-      <c r="A22" s="2" t="inlineStr">
-        <is>
-          <t>phe_fingertips_92901</t>
-        </is>
-      </c>
-      <c r="B22" s="2" t="inlineStr">
-        <is>
-          <t>Life expectancy inequality at birth by local authority in the South West, 2022 - 24</t>
-        </is>
-      </c>
-      <c r="C22" s="2" t="inlineStr">
-        <is>
-          <t>Fingertips — Inequality in life expectancy at birth (Slope Index of Inequality), Indicator 92901</t>
-        </is>
-      </c>
-      <c r="D22" s="2" t="inlineStr">
-        <is>
-          <t>https://fingertips.phe.org.uk/indicator-details/90/indicator/92901</t>
-        </is>
-      </c>
-      <c r="E22" s="2" t="inlineStr">
-        <is>
-          <t>2022 - 24</t>
-        </is>
-      </c>
-      <c r="F22" s="2" t="inlineStr">
-        <is>
-          <t>three_year_period</t>
-        </is>
-      </c>
-      <c r="G22" s="2" t="n">
-        <v>2022</v>
-      </c>
-      <c r="H22" s="2" t="inlineStr">
-        <is>
-          <t>Swindon</t>
-        </is>
-      </c>
-      <c r="I22" s="2" t="inlineStr">
-        <is>
-          <t>E06000030</t>
-        </is>
-      </c>
-      <c r="J22" s="2" t="inlineStr">
-        <is>
-          <t>Swindon</t>
-        </is>
-      </c>
-      <c r="K22" s="2" t="inlineStr">
-        <is>
-          <t>E06000030</t>
-        </is>
-      </c>
-      <c r="L22" s="2" t="inlineStr">
-        <is>
-          <t>local_authority</t>
-        </is>
-      </c>
-      <c r="M22" s="2" t="inlineStr">
-        <is>
-          <t>life_expectancy_inequality_sii_birth</t>
-        </is>
-      </c>
-      <c r="N22" s="2" t="inlineStr">
-        <is>
-          <t>Slope index of inequality in life expectancy at birth</t>
-        </is>
-      </c>
-      <c r="O22" s="2" t="n">
-        <v>5.67937352872535</v>
-      </c>
-      <c r="P22" s="2" t="inlineStr">
-        <is>
-          <t>years</t>
-        </is>
-      </c>
-      <c r="Q22" s="2" t="inlineStr"/>
-      <c r="R22" s="2" t="inlineStr"/>
-      <c r="S22" s="2" t="inlineStr"/>
-      <c r="T22" s="2" t="inlineStr"/>
-      <c r="U22" s="2" t="inlineStr"/>
-      <c r="V22" s="2" t="n">
-        <v>4.23304060137117</v>
-      </c>
-      <c r="W22" s="2" t="n">
-        <v>7.12145672576508</v>
-      </c>
-      <c r="X22" s="2" t="inlineStr"/>
-      <c r="Y22" s="2" t="inlineStr">
-        <is>
-          <t>Female</t>
-        </is>
-      </c>
-      <c r="Z22" s="2" t="inlineStr"/>
-      <c r="AA22" s="2" t="inlineStr"/>
-      <c r="AB22" s="2" t="inlineStr"/>
-      <c r="AC22" s="2" t="inlineStr">
-        <is>
-          <t>{"sex": "Female"}</t>
-        </is>
-      </c>
-      <c r="AD22" s="2" t="inlineStr">
-        <is>
-          <t>Fingertips Indicator 92901</t>
-        </is>
-      </c>
-      <c r="AE22" s="2" t="inlineStr">
-        <is>
-          <t>SII value</t>
-        </is>
-      </c>
-      <c r="AF22" s="2" t="inlineStr"/>
-      <c r="AG22" s="2" t="inlineStr">
-        <is>
-          <t>Direct</t>
-        </is>
-      </c>
-      <c r="AH22" s="2" t="inlineStr"/>
-      <c r="AI22" s="2" t="inlineStr"/>
-      <c r="AJ22" s="2" t="inlineStr">
-        <is>
-          <t>2026-07-22</t>
-        </is>
-      </c>
-    </row>
-    <row r="23">
-      <c r="A23" s="2" t="inlineStr">
-        <is>
-          <t>phe_fingertips_92901</t>
-        </is>
-      </c>
-      <c r="B23" s="2" t="inlineStr">
-        <is>
-          <t>Life expectancy inequality at birth by local authority in the South West, 2022 - 24</t>
-        </is>
-      </c>
-      <c r="C23" s="2" t="inlineStr">
-        <is>
-          <t>Fingertips — Inequality in life expectancy at birth (Slope Index of Inequality), Indicator 92901</t>
-        </is>
-      </c>
-      <c r="D23" s="2" t="inlineStr">
-        <is>
-          <t>https://fingertips.phe.org.uk/indicator-details/90/indicator/92901</t>
-        </is>
-      </c>
-      <c r="E23" s="2" t="inlineStr">
-        <is>
-          <t>2022 - 24</t>
-        </is>
-      </c>
-      <c r="F23" s="2" t="inlineStr">
-        <is>
-          <t>three_year_period</t>
-        </is>
-      </c>
-      <c r="G23" s="2" t="n">
-        <v>2022</v>
-      </c>
-      <c r="H23" s="2" t="inlineStr">
-        <is>
-          <t>Swindon</t>
-        </is>
-      </c>
-      <c r="I23" s="2" t="inlineStr">
-        <is>
-          <t>E06000030</t>
-        </is>
-      </c>
-      <c r="J23" s="2" t="inlineStr">
-        <is>
-          <t>Swindon</t>
-        </is>
-      </c>
-      <c r="K23" s="2" t="inlineStr">
-        <is>
-          <t>E06000030</t>
-        </is>
-      </c>
-      <c r="L23" s="2" t="inlineStr">
-        <is>
-          <t>local_authority</t>
-        </is>
-      </c>
-      <c r="M23" s="2" t="inlineStr">
-        <is>
-          <t>life_expectancy_inequality_sii_birth</t>
-        </is>
-      </c>
-      <c r="N23" s="2" t="inlineStr">
-        <is>
-          <t>Slope index of inequality in life expectancy at birth</t>
-        </is>
-      </c>
-      <c r="O23" s="2" t="n">
-        <v>81.0495001459274</v>
-      </c>
-      <c r="P23" s="2" t="inlineStr">
-        <is>
-          <t>years</t>
-        </is>
-      </c>
-      <c r="Q23" s="2" t="inlineStr"/>
-      <c r="R23" s="2" t="inlineStr"/>
-      <c r="S23" s="2" t="inlineStr"/>
-      <c r="T23" s="2" t="inlineStr"/>
-      <c r="U23" s="2" t="inlineStr"/>
-      <c r="V23" s="2" t="n"/>
-      <c r="W23" s="2" t="n"/>
-      <c r="X23" s="2" t="inlineStr"/>
-      <c r="Y23" s="2" t="inlineStr">
-        <is>
-          <t>Female</t>
-        </is>
-      </c>
-      <c r="Z23" s="2" t="inlineStr"/>
-      <c r="AA23" s="2" t="inlineStr"/>
-      <c r="AB23" s="2" t="inlineStr"/>
-      <c r="AC23" s="2" t="inlineStr">
-        <is>
-          <t>{"sex": "Female"}</t>
-        </is>
-      </c>
-      <c r="AD23" s="2" t="inlineStr">
-        <is>
-          <t>Fingertips Indicator 92901</t>
-        </is>
-      </c>
-      <c r="AE23" s="2" t="inlineStr">
-        <is>
-          <t>Limits for SII regression charts</t>
-        </is>
-      </c>
-      <c r="AF23" s="2" t="inlineStr"/>
-      <c r="AG23" s="2" t="inlineStr">
-        <is>
-          <t>Direct</t>
-        </is>
-      </c>
-      <c r="AH23" s="2" t="inlineStr"/>
-      <c r="AI23" s="2" t="inlineStr"/>
-      <c r="AJ23" s="2" t="inlineStr">
-        <is>
-          <t>2026-07-22</t>
-        </is>
-      </c>
-    </row>
-    <row r="24">
-      <c r="A24" s="2" t="inlineStr">
-        <is>
-          <t>phe_fingertips_92901</t>
-        </is>
-      </c>
-      <c r="B24" s="2" t="inlineStr">
-        <is>
-          <t>Life expectancy inequality at birth by local authority in the South West, 2022 - 24</t>
-        </is>
-      </c>
-      <c r="C24" s="2" t="inlineStr">
-        <is>
-          <t>Fingertips — Inequality in life expectancy at birth (Slope Index of Inequality), Indicator 92901</t>
-        </is>
-      </c>
-      <c r="D24" s="2" t="inlineStr">
-        <is>
-          <t>https://fingertips.phe.org.uk/indicator-details/90/indicator/92901</t>
-        </is>
-      </c>
-      <c r="E24" s="2" t="inlineStr">
-        <is>
-          <t>2022 - 24</t>
-        </is>
-      </c>
-      <c r="F24" s="2" t="inlineStr">
-        <is>
-          <t>three_year_period</t>
-        </is>
-      </c>
-      <c r="G24" s="2" t="n">
-        <v>2022</v>
-      </c>
-      <c r="H24" s="2" t="inlineStr">
-        <is>
-          <t>Swindon</t>
-        </is>
-      </c>
-      <c r="I24" s="2" t="inlineStr">
-        <is>
-          <t>E06000030</t>
-        </is>
-      </c>
-      <c r="J24" s="2" t="inlineStr">
-        <is>
-          <t>Swindon</t>
-        </is>
-      </c>
-      <c r="K24" s="2" t="inlineStr">
-        <is>
-          <t>E06000030</t>
-        </is>
-      </c>
-      <c r="L24" s="2" t="inlineStr">
-        <is>
-          <t>local_authority</t>
-        </is>
-      </c>
-      <c r="M24" s="2" t="inlineStr">
-        <is>
-          <t>life_expectancy_inequality_sii_birth</t>
-        </is>
-      </c>
-      <c r="N24" s="2" t="inlineStr">
-        <is>
-          <t>Slope index of inequality in life expectancy at birth</t>
-        </is>
-      </c>
-      <c r="O24" s="2" t="n">
-        <v>9.97135672505077</v>
-      </c>
-      <c r="P24" s="2" t="inlineStr">
-        <is>
-          <t>years</t>
-        </is>
-      </c>
-      <c r="Q24" s="2" t="inlineStr"/>
-      <c r="R24" s="2" t="inlineStr"/>
-      <c r="S24" s="2" t="inlineStr"/>
-      <c r="T24" s="2" t="inlineStr"/>
-      <c r="U24" s="2" t="inlineStr"/>
-      <c r="V24" s="2" t="n">
-        <v>8.47354893144897</v>
-      </c>
-      <c r="W24" s="2" t="n">
-        <v>11.4659628814125</v>
-      </c>
-      <c r="X24" s="2" t="inlineStr"/>
-      <c r="Y24" s="2" t="inlineStr">
-        <is>
-          <t>Male</t>
-        </is>
-      </c>
-      <c r="Z24" s="2" t="inlineStr"/>
-      <c r="AA24" s="2" t="inlineStr"/>
-      <c r="AB24" s="2" t="inlineStr"/>
-      <c r="AC24" s="2" t="inlineStr">
-        <is>
-          <t>{"sex": "Male"}</t>
-        </is>
-      </c>
-      <c r="AD24" s="2" t="inlineStr">
-        <is>
-          <t>Fingertips Indicator 92901</t>
-        </is>
-      </c>
-      <c r="AE24" s="2" t="inlineStr">
-        <is>
-          <t>SII value</t>
-        </is>
-      </c>
-      <c r="AF24" s="2" t="inlineStr"/>
-      <c r="AG24" s="2" t="inlineStr">
-        <is>
-          <t>Direct</t>
-        </is>
-      </c>
-      <c r="AH24" s="2" t="inlineStr"/>
-      <c r="AI24" s="2" t="inlineStr"/>
-      <c r="AJ24" s="2" t="inlineStr">
-        <is>
-          <t>2026-07-22</t>
-        </is>
-      </c>
-    </row>
-    <row r="25">
-      <c r="A25" s="2" t="inlineStr">
-        <is>
-          <t>phe_fingertips_92901</t>
-        </is>
-      </c>
-      <c r="B25" s="2" t="inlineStr">
-        <is>
-          <t>Life expectancy inequality at birth by local authority in the South West, 2022 - 24</t>
-        </is>
-      </c>
-      <c r="C25" s="2" t="inlineStr">
-        <is>
-          <t>Fingertips — Inequality in life expectancy at birth (Slope Index of Inequality), Indicator 92901</t>
-        </is>
-      </c>
-      <c r="D25" s="2" t="inlineStr">
-        <is>
-          <t>https://fingertips.phe.org.uk/indicator-details/90/indicator/92901</t>
-        </is>
-      </c>
-      <c r="E25" s="2" t="inlineStr">
-        <is>
-          <t>2022 - 24</t>
-        </is>
-      </c>
-      <c r="F25" s="2" t="inlineStr">
-        <is>
-          <t>three_year_period</t>
-        </is>
-      </c>
-      <c r="G25" s="2" t="n">
-        <v>2022</v>
-      </c>
-      <c r="H25" s="2" t="inlineStr">
-        <is>
-          <t>Swindon</t>
-        </is>
-      </c>
-      <c r="I25" s="2" t="inlineStr">
-        <is>
-          <t>E06000030</t>
-        </is>
-      </c>
-      <c r="J25" s="2" t="inlineStr">
-        <is>
-          <t>Swindon</t>
-        </is>
-      </c>
-      <c r="K25" s="2" t="inlineStr">
-        <is>
-          <t>E06000030</t>
-        </is>
-      </c>
-      <c r="L25" s="2" t="inlineStr">
-        <is>
-          <t>local_authority</t>
-        </is>
-      </c>
-      <c r="M25" s="2" t="inlineStr">
-        <is>
-          <t>life_expectancy_inequality_sii_birth</t>
-        </is>
-      </c>
-      <c r="N25" s="2" t="inlineStr">
-        <is>
-          <t>Slope index of inequality in life expectancy at birth</t>
-        </is>
-      </c>
-      <c r="O25" s="2" t="n">
-        <v>75.02292616219439</v>
-      </c>
-      <c r="P25" s="2" t="inlineStr">
-        <is>
-          <t>years</t>
-        </is>
-      </c>
-      <c r="Q25" s="2" t="inlineStr"/>
-      <c r="R25" s="2" t="inlineStr"/>
-      <c r="S25" s="2" t="inlineStr"/>
-      <c r="T25" s="2" t="inlineStr"/>
-      <c r="U25" s="2" t="inlineStr"/>
-      <c r="V25" s="2" t="n"/>
-      <c r="W25" s="2" t="n"/>
-      <c r="X25" s="2" t="inlineStr"/>
-      <c r="Y25" s="2" t="inlineStr">
-        <is>
-          <t>Male</t>
-        </is>
-      </c>
-      <c r="Z25" s="2" t="inlineStr"/>
-      <c r="AA25" s="2" t="inlineStr"/>
-      <c r="AB25" s="2" t="inlineStr"/>
-      <c r="AC25" s="2" t="inlineStr">
-        <is>
-          <t>{"sex": "Male"}</t>
-        </is>
-      </c>
-      <c r="AD25" s="2" t="inlineStr">
-        <is>
-          <t>Fingertips Indicator 92901</t>
-        </is>
-      </c>
-      <c r="AE25" s="2" t="inlineStr">
-        <is>
-          <t>Limits for SII regression charts</t>
-        </is>
-      </c>
-      <c r="AF25" s="2" t="inlineStr"/>
-      <c r="AG25" s="2" t="inlineStr">
-        <is>
-          <t>Direct</t>
-        </is>
-      </c>
-      <c r="AH25" s="2" t="inlineStr"/>
-      <c r="AI25" s="2" t="inlineStr"/>
-      <c r="AJ25" s="2" t="inlineStr">
-        <is>
-          <t>2026-07-22</t>
-        </is>
-      </c>
-    </row>
-    <row r="26">
-      <c r="A26" s="2" t="inlineStr">
-        <is>
-          <t>phe_fingertips_92901</t>
-        </is>
-      </c>
-      <c r="B26" s="2" t="inlineStr">
-        <is>
-          <t>Life expectancy inequality at birth by local authority in the South West, 2022 - 24</t>
-        </is>
-      </c>
-      <c r="C26" s="2" t="inlineStr">
-        <is>
-          <t>Fingertips — Inequality in life expectancy at birth (Slope Index of Inequality), Indicator 92901</t>
-        </is>
-      </c>
-      <c r="D26" s="2" t="inlineStr">
-        <is>
-          <t>https://fingertips.phe.org.uk/indicator-details/90/indicator/92901</t>
-        </is>
-      </c>
-      <c r="E26" s="2" t="inlineStr">
-        <is>
-          <t>2022 - 24</t>
-        </is>
-      </c>
-      <c r="F26" s="2" t="inlineStr">
-        <is>
-          <t>three_year_period</t>
-        </is>
-      </c>
-      <c r="G26" s="2" t="n">
-        <v>2022</v>
-      </c>
-      <c r="H26" s="2" t="inlineStr">
-        <is>
-          <t>Wiltshire</t>
-        </is>
-      </c>
-      <c r="I26" s="2" t="inlineStr">
-        <is>
-          <t>E06000054</t>
-        </is>
-      </c>
-      <c r="J26" s="2" t="inlineStr">
-        <is>
-          <t>Wiltshire</t>
-        </is>
-      </c>
-      <c r="K26" s="2" t="inlineStr">
-        <is>
-          <t>E06000054</t>
-        </is>
-      </c>
-      <c r="L26" s="2" t="inlineStr">
-        <is>
-          <t>local_authority</t>
-        </is>
-      </c>
-      <c r="M26" s="2" t="inlineStr">
-        <is>
-          <t>life_expectancy_inequality_sii_birth</t>
-        </is>
-      </c>
-      <c r="N26" s="2" t="inlineStr">
-        <is>
-          <t>Slope index of inequality in life expectancy at birth</t>
-        </is>
-      </c>
-      <c r="O26" s="2" t="n">
-        <v>3.68786604792967</v>
-      </c>
-      <c r="P26" s="2" t="inlineStr">
-        <is>
-          <t>years</t>
-        </is>
-      </c>
-      <c r="Q26" s="2" t="inlineStr"/>
-      <c r="R26" s="2" t="inlineStr"/>
-      <c r="S26" s="2" t="inlineStr"/>
-      <c r="T26" s="2" t="inlineStr"/>
-      <c r="U26" s="2" t="inlineStr"/>
-      <c r="V26" s="2" t="n">
-        <v>2.74496766069945</v>
-      </c>
-      <c r="W26" s="2" t="n">
-        <v>4.62779265274191</v>
-      </c>
-      <c r="X26" s="2" t="inlineStr"/>
-      <c r="Y26" s="2" t="inlineStr">
-        <is>
-          <t>Female</t>
-        </is>
-      </c>
-      <c r="Z26" s="2" t="inlineStr"/>
-      <c r="AA26" s="2" t="inlineStr"/>
-      <c r="AB26" s="2" t="inlineStr"/>
-      <c r="AC26" s="2" t="inlineStr">
-        <is>
-          <t>{"sex": "Female"}</t>
-        </is>
-      </c>
-      <c r="AD26" s="2" t="inlineStr">
-        <is>
-          <t>Fingertips Indicator 92901</t>
-        </is>
-      </c>
-      <c r="AE26" s="2" t="inlineStr">
-        <is>
-          <t>SII value</t>
-        </is>
-      </c>
-      <c r="AF26" s="2" t="inlineStr"/>
-      <c r="AG26" s="2" t="inlineStr">
-        <is>
-          <t>Direct</t>
-        </is>
-      </c>
-      <c r="AH26" s="2" t="inlineStr"/>
-      <c r="AI26" s="2" t="inlineStr"/>
-      <c r="AJ26" s="2" t="inlineStr">
-        <is>
-          <t>2026-07-22</t>
-        </is>
-      </c>
-    </row>
-    <row r="27">
-      <c r="A27" s="2" t="inlineStr">
-        <is>
-          <t>phe_fingertips_92901</t>
-        </is>
-      </c>
-      <c r="B27" s="2" t="inlineStr">
-        <is>
-          <t>Life expectancy inequality at birth by local authority in the South West, 2022 - 24</t>
-        </is>
-      </c>
-      <c r="C27" s="2" t="inlineStr">
-        <is>
-          <t>Fingertips — Inequality in life expectancy at birth (Slope Index of Inequality), Indicator 92901</t>
-        </is>
-      </c>
-      <c r="D27" s="2" t="inlineStr">
-        <is>
-          <t>https://fingertips.phe.org.uk/indicator-details/90/indicator/92901</t>
-        </is>
-      </c>
-      <c r="E27" s="2" t="inlineStr">
-        <is>
-          <t>2022 - 24</t>
-        </is>
-      </c>
-      <c r="F27" s="2" t="inlineStr">
-        <is>
-          <t>three_year_period</t>
-        </is>
-      </c>
-      <c r="G27" s="2" t="n">
-        <v>2022</v>
-      </c>
-      <c r="H27" s="2" t="inlineStr">
-        <is>
-          <t>Wiltshire</t>
-        </is>
-      </c>
-      <c r="I27" s="2" t="inlineStr">
-        <is>
-          <t>E06000054</t>
-        </is>
-      </c>
-      <c r="J27" s="2" t="inlineStr">
-        <is>
-          <t>Wiltshire</t>
-        </is>
-      </c>
-      <c r="K27" s="2" t="inlineStr">
-        <is>
-          <t>E06000054</t>
-        </is>
-      </c>
-      <c r="L27" s="2" t="inlineStr">
-        <is>
-          <t>local_authority</t>
-        </is>
-      </c>
-      <c r="M27" s="2" t="inlineStr">
-        <is>
-          <t>life_expectancy_inequality_sii_birth</t>
-        </is>
-      </c>
-      <c r="N27" s="2" t="inlineStr">
-        <is>
-          <t>Slope index of inequality in life expectancy at birth</t>
-        </is>
-      </c>
-      <c r="O27" s="2" t="n">
-        <v>82.88747088685319</v>
-      </c>
-      <c r="P27" s="2" t="inlineStr">
-        <is>
-          <t>years</t>
-        </is>
-      </c>
-      <c r="Q27" s="2" t="inlineStr"/>
-      <c r="R27" s="2" t="inlineStr"/>
-      <c r="S27" s="2" t="inlineStr"/>
-      <c r="T27" s="2" t="inlineStr"/>
-      <c r="U27" s="2" t="inlineStr"/>
-      <c r="V27" s="2" t="n"/>
-      <c r="W27" s="2" t="n"/>
-      <c r="X27" s="2" t="inlineStr"/>
-      <c r="Y27" s="2" t="inlineStr">
-        <is>
-          <t>Female</t>
-        </is>
-      </c>
-      <c r="Z27" s="2" t="inlineStr"/>
-      <c r="AA27" s="2" t="inlineStr"/>
-      <c r="AB27" s="2" t="inlineStr"/>
-      <c r="AC27" s="2" t="inlineStr">
-        <is>
-          <t>{"sex": "Female"}</t>
-        </is>
-      </c>
-      <c r="AD27" s="2" t="inlineStr">
-        <is>
-          <t>Fingertips Indicator 92901</t>
-        </is>
-      </c>
-      <c r="AE27" s="2" t="inlineStr">
-        <is>
-          <t>Limits for SII regression charts</t>
-        </is>
-      </c>
-      <c r="AF27" s="2" t="inlineStr"/>
-      <c r="AG27" s="2" t="inlineStr">
-        <is>
-          <t>Direct</t>
-        </is>
-      </c>
-      <c r="AH27" s="2" t="inlineStr"/>
-      <c r="AI27" s="2" t="inlineStr"/>
-      <c r="AJ27" s="2" t="inlineStr">
-        <is>
-          <t>2026-07-22</t>
-        </is>
-      </c>
-    </row>
-    <row r="28">
-      <c r="A28" s="2" t="inlineStr">
-        <is>
-          <t>phe_fingertips_92901</t>
-        </is>
-      </c>
-      <c r="B28" s="2" t="inlineStr">
-        <is>
-          <t>Life expectancy inequality at birth by local authority in the South West, 2022 - 24</t>
-        </is>
-      </c>
-      <c r="C28" s="2" t="inlineStr">
-        <is>
-          <t>Fingertips — Inequality in life expectancy at birth (Slope Index of Inequality), Indicator 92901</t>
-        </is>
-      </c>
-      <c r="D28" s="2" t="inlineStr">
-        <is>
-          <t>https://fingertips.phe.org.uk/indicator-details/90/indicator/92901</t>
-        </is>
-      </c>
-      <c r="E28" s="2" t="inlineStr">
-        <is>
-          <t>2022 - 24</t>
-        </is>
-      </c>
-      <c r="F28" s="2" t="inlineStr">
-        <is>
-          <t>three_year_period</t>
-        </is>
-      </c>
-      <c r="G28" s="2" t="n">
-        <v>2022</v>
-      </c>
-      <c r="H28" s="2" t="inlineStr">
-        <is>
-          <t>Wiltshire</t>
-        </is>
-      </c>
-      <c r="I28" s="2" t="inlineStr">
-        <is>
-          <t>E06000054</t>
-        </is>
-      </c>
-      <c r="J28" s="2" t="inlineStr">
-        <is>
-          <t>Wiltshire</t>
-        </is>
-      </c>
-      <c r="K28" s="2" t="inlineStr">
-        <is>
-          <t>E06000054</t>
-        </is>
-      </c>
-      <c r="L28" s="2" t="inlineStr">
-        <is>
-          <t>local_authority</t>
-        </is>
-      </c>
-      <c r="M28" s="2" t="inlineStr">
-        <is>
-          <t>life_expectancy_inequality_sii_birth</t>
-        </is>
-      </c>
-      <c r="N28" s="2" t="inlineStr">
-        <is>
-          <t>Slope index of inequality in life expectancy at birth</t>
-        </is>
-      </c>
-      <c r="O28" s="2" t="n">
-        <v>4.91994895362696</v>
-      </c>
-      <c r="P28" s="2" t="inlineStr">
-        <is>
-          <t>years</t>
-        </is>
-      </c>
-      <c r="Q28" s="2" t="inlineStr"/>
-      <c r="R28" s="2" t="inlineStr"/>
-      <c r="S28" s="2" t="inlineStr"/>
-      <c r="T28" s="2" t="inlineStr"/>
-      <c r="U28" s="2" t="inlineStr"/>
-      <c r="V28" s="2" t="n">
-        <v>3.92504759854335</v>
-      </c>
-      <c r="W28" s="2" t="n">
-        <v>5.91316284510629</v>
-      </c>
-      <c r="X28" s="2" t="inlineStr"/>
-      <c r="Y28" s="2" t="inlineStr">
-        <is>
-          <t>Male</t>
-        </is>
-      </c>
-      <c r="Z28" s="2" t="inlineStr"/>
-      <c r="AA28" s="2" t="inlineStr"/>
-      <c r="AB28" s="2" t="inlineStr"/>
-      <c r="AC28" s="2" t="inlineStr">
-        <is>
-          <t>{"sex": "Male"}</t>
-        </is>
-      </c>
-      <c r="AD28" s="2" t="inlineStr">
-        <is>
-          <t>Fingertips Indicator 92901</t>
-        </is>
-      </c>
-      <c r="AE28" s="2" t="inlineStr">
-        <is>
-          <t>SII value</t>
-        </is>
-      </c>
-      <c r="AF28" s="2" t="inlineStr"/>
-      <c r="AG28" s="2" t="inlineStr">
-        <is>
-          <t>Direct</t>
-        </is>
-      </c>
-      <c r="AH28" s="2" t="inlineStr"/>
-      <c r="AI28" s="2" t="inlineStr"/>
-      <c r="AJ28" s="2" t="inlineStr">
-        <is>
-          <t>2026-07-22</t>
-        </is>
-      </c>
-    </row>
-    <row r="29">
-      <c r="A29" s="2" t="inlineStr">
-        <is>
-          <t>phe_fingertips_92901</t>
-        </is>
-      </c>
-      <c r="B29" s="2" t="inlineStr">
-        <is>
-          <t>Life expectancy inequality at birth by local authority in the South West, 2022 - 24</t>
-        </is>
-      </c>
-      <c r="C29" s="2" t="inlineStr">
-        <is>
-          <t>Fingertips — Inequality in life expectancy at birth (Slope Index of Inequality), Indicator 92901</t>
-        </is>
-      </c>
-      <c r="D29" s="2" t="inlineStr">
-        <is>
-          <t>https://fingertips.phe.org.uk/indicator-details/90/indicator/92901</t>
-        </is>
-      </c>
-      <c r="E29" s="2" t="inlineStr">
-        <is>
-          <t>2022 - 24</t>
-        </is>
-      </c>
-      <c r="F29" s="2" t="inlineStr">
-        <is>
-          <t>three_year_period</t>
-        </is>
-      </c>
-      <c r="G29" s="2" t="n">
-        <v>2022</v>
-      </c>
-      <c r="H29" s="2" t="inlineStr">
-        <is>
-          <t>Wiltshire</t>
-        </is>
-      </c>
-      <c r="I29" s="2" t="inlineStr">
-        <is>
-          <t>E06000054</t>
-        </is>
-      </c>
-      <c r="J29" s="2" t="inlineStr">
-        <is>
-          <t>Wiltshire</t>
-        </is>
-      </c>
-      <c r="K29" s="2" t="inlineStr">
-        <is>
-          <t>E06000054</t>
-        </is>
-      </c>
-      <c r="L29" s="2" t="inlineStr">
-        <is>
-          <t>local_authority</t>
-        </is>
-      </c>
-      <c r="M29" s="2" t="inlineStr">
-        <is>
-          <t>life_expectancy_inequality_sii_birth</t>
-        </is>
-      </c>
-      <c r="N29" s="2" t="inlineStr">
-        <is>
-          <t>Slope index of inequality in life expectancy at birth</t>
-        </is>
-      </c>
-      <c r="O29" s="2" t="n">
-        <v>78.878214659915</v>
-      </c>
-      <c r="P29" s="2" t="inlineStr">
-        <is>
-          <t>years</t>
-        </is>
-      </c>
-      <c r="Q29" s="2" t="inlineStr"/>
-      <c r="R29" s="2" t="inlineStr"/>
-      <c r="S29" s="2" t="inlineStr"/>
-      <c r="T29" s="2" t="inlineStr"/>
-      <c r="U29" s="2" t="inlineStr"/>
-      <c r="V29" s="2" t="n"/>
-      <c r="W29" s="2" t="n"/>
-      <c r="X29" s="2" t="inlineStr"/>
-      <c r="Y29" s="2" t="inlineStr">
-        <is>
-          <t>Male</t>
-        </is>
-      </c>
-      <c r="Z29" s="2" t="inlineStr"/>
-      <c r="AA29" s="2" t="inlineStr"/>
-      <c r="AB29" s="2" t="inlineStr"/>
-      <c r="AC29" s="2" t="inlineStr">
-        <is>
-          <t>{"sex": "Male"}</t>
-        </is>
-      </c>
-      <c r="AD29" s="2" t="inlineStr">
-        <is>
-          <t>Fingertips Indicator 92901</t>
-        </is>
-      </c>
-      <c r="AE29" s="2" t="inlineStr">
-        <is>
-          <t>Limits for SII regression charts</t>
-        </is>
-      </c>
-      <c r="AF29" s="2" t="inlineStr"/>
-      <c r="AG29" s="2" t="inlineStr">
-        <is>
-          <t>Direct</t>
-        </is>
-      </c>
-      <c r="AH29" s="2" t="inlineStr"/>
-      <c r="AI29" s="2" t="inlineStr"/>
-      <c r="AJ29" s="2" t="inlineStr">
-        <is>
-          <t>2026-07-22</t>
-        </is>
-      </c>
-    </row>
-    <row r="30">
-      <c r="A30" s="2" t="inlineStr">
-        <is>
-          <t>phe_fingertips_92901</t>
-        </is>
-      </c>
-      <c r="B30" s="2" t="inlineStr">
-        <is>
-          <t>Life expectancy inequality at birth by local authority in the South West, 2022 - 24</t>
-        </is>
-      </c>
-      <c r="C30" s="2" t="inlineStr">
-        <is>
-          <t>Fingertips — Inequality in life expectancy at birth (Slope Index of Inequality), Indicator 92901</t>
-        </is>
-      </c>
-      <c r="D30" s="2" t="inlineStr">
-        <is>
-          <t>https://fingertips.phe.org.uk/indicator-details/90/indicator/92901</t>
-        </is>
-      </c>
-      <c r="E30" s="2" t="inlineStr">
-        <is>
-          <t>2022 - 24</t>
-        </is>
-      </c>
-      <c r="F30" s="2" t="inlineStr">
-        <is>
-          <t>three_year_period</t>
-        </is>
-      </c>
-      <c r="G30" s="2" t="n">
-        <v>2022</v>
-      </c>
-      <c r="H30" s="2" t="inlineStr">
-        <is>
-          <t>England</t>
-        </is>
-      </c>
-      <c r="I30" s="2" t="inlineStr">
-        <is>
-          <t>E92000001</t>
-        </is>
-      </c>
-      <c r="J30" s="2" t="inlineStr">
-        <is>
-          <t>England</t>
-        </is>
-      </c>
-      <c r="K30" s="2" t="inlineStr">
-        <is>
-          <t>E92000001</t>
-        </is>
-      </c>
-      <c r="L30" s="2" t="inlineStr">
-        <is>
-          <t>country</t>
-        </is>
-      </c>
-      <c r="M30" s="2" t="inlineStr">
-        <is>
-          <t>life_expectancy_inequality_sii_birth</t>
-        </is>
-      </c>
-      <c r="N30" s="2" t="inlineStr">
-        <is>
-          <t>Slope index of inequality in life expectancy at birth</t>
-        </is>
-      </c>
-      <c r="O30" s="2" t="n">
-        <v>8.029185211892139</v>
-      </c>
-      <c r="P30" s="2" t="inlineStr">
-        <is>
-          <t>years</t>
-        </is>
-      </c>
-      <c r="Q30" s="2" t="inlineStr"/>
-      <c r="R30" s="2" t="inlineStr"/>
-      <c r="S30" s="2" t="inlineStr"/>
-      <c r="T30" s="2" t="inlineStr"/>
-      <c r="U30" s="2" t="inlineStr"/>
-      <c r="V30" s="2" t="n">
-        <v>7.9351805783358</v>
-      </c>
-      <c r="W30" s="2" t="n">
-        <v>8.12327840388291</v>
-      </c>
-      <c r="X30" s="2" t="inlineStr"/>
-      <c r="Y30" s="2" t="inlineStr">
-        <is>
-          <t>Female</t>
-        </is>
-      </c>
-      <c r="Z30" s="2" t="inlineStr"/>
-      <c r="AA30" s="2" t="inlineStr"/>
-      <c r="AB30" s="2" t="inlineStr"/>
-      <c r="AC30" s="2" t="inlineStr">
-        <is>
-          <t>{"sex": "Female"}</t>
-        </is>
-      </c>
-      <c r="AD30" s="2" t="inlineStr">
-        <is>
-          <t>Fingertips Indicator 92901</t>
-        </is>
-      </c>
-      <c r="AE30" s="2" t="inlineStr">
-        <is>
-          <t>SII value</t>
-        </is>
-      </c>
-      <c r="AF30" s="2" t="inlineStr"/>
-      <c r="AG30" s="2" t="inlineStr">
-        <is>
-          <t>Direct</t>
-        </is>
-      </c>
-      <c r="AH30" s="2" t="inlineStr"/>
-      <c r="AI30" s="2" t="inlineStr"/>
-      <c r="AJ30" s="2" t="inlineStr">
-        <is>
-          <t>2026-07-22</t>
-        </is>
-      </c>
-    </row>
-    <row r="31">
-      <c r="A31" s="2" t="inlineStr">
-        <is>
-          <t>phe_fingertips_92901</t>
-        </is>
-      </c>
-      <c r="B31" s="2" t="inlineStr">
-        <is>
-          <t>Life expectancy inequality at birth by local authority in the South West, 2022 - 24</t>
-        </is>
-      </c>
-      <c r="C31" s="2" t="inlineStr">
-        <is>
-          <t>Fingertips — Inequality in life expectancy at birth (Slope Index of Inequality), Indicator 92901</t>
-        </is>
-      </c>
-      <c r="D31" s="2" t="inlineStr">
-        <is>
-          <t>https://fingertips.phe.org.uk/indicator-details/90/indicator/92901</t>
-        </is>
-      </c>
-      <c r="E31" s="2" t="inlineStr">
-        <is>
-          <t>2022 - 24</t>
-        </is>
-      </c>
-      <c r="F31" s="2" t="inlineStr">
-        <is>
-          <t>three_year_period</t>
-        </is>
-      </c>
-      <c r="G31" s="2" t="n">
-        <v>2022</v>
-      </c>
-      <c r="H31" s="2" t="inlineStr">
-        <is>
-          <t>England</t>
-        </is>
-      </c>
-      <c r="I31" s="2" t="inlineStr">
-        <is>
-          <t>E92000001</t>
-        </is>
-      </c>
-      <c r="J31" s="2" t="inlineStr">
-        <is>
-          <t>England</t>
-        </is>
-      </c>
-      <c r="K31" s="2" t="inlineStr">
-        <is>
-          <t>E92000001</t>
-        </is>
-      </c>
-      <c r="L31" s="2" t="inlineStr">
-        <is>
-          <t>country</t>
-        </is>
-      </c>
-      <c r="M31" s="2" t="inlineStr">
-        <is>
-          <t>life_expectancy_inequality_sii_birth</t>
-        </is>
-      </c>
-      <c r="N31" s="2" t="inlineStr">
-        <is>
-          <t>Slope index of inequality in life expectancy at birth</t>
-        </is>
-      </c>
-      <c r="O31" s="2" t="n">
-        <v>79.1748961928772</v>
-      </c>
-      <c r="P31" s="2" t="inlineStr">
-        <is>
-          <t>years</t>
-        </is>
-      </c>
-      <c r="Q31" s="2" t="inlineStr"/>
-      <c r="R31" s="2" t="inlineStr"/>
-      <c r="S31" s="2" t="inlineStr"/>
-      <c r="T31" s="2" t="inlineStr"/>
-      <c r="U31" s="2" t="inlineStr"/>
-      <c r="V31" s="2" t="n"/>
-      <c r="W31" s="2" t="n"/>
-      <c r="X31" s="2" t="inlineStr"/>
-      <c r="Y31" s="2" t="inlineStr">
-        <is>
-          <t>Female</t>
-        </is>
-      </c>
-      <c r="Z31" s="2" t="inlineStr"/>
-      <c r="AA31" s="2" t="inlineStr"/>
-      <c r="AB31" s="2" t="inlineStr"/>
-      <c r="AC31" s="2" t="inlineStr">
-        <is>
-          <t>{"sex": "Female"}</t>
-        </is>
-      </c>
-      <c r="AD31" s="2" t="inlineStr">
-        <is>
-          <t>Fingertips Indicator 92901</t>
-        </is>
-      </c>
-      <c r="AE31" s="2" t="inlineStr">
-        <is>
-          <t>Limits for SII regression charts</t>
-        </is>
-      </c>
-      <c r="AF31" s="2" t="inlineStr"/>
-      <c r="AG31" s="2" t="inlineStr">
-        <is>
-          <t>Direct</t>
-        </is>
-      </c>
-      <c r="AH31" s="2" t="inlineStr"/>
-      <c r="AI31" s="2" t="inlineStr"/>
-      <c r="AJ31" s="2" t="inlineStr">
-        <is>
-          <t>2026-07-22</t>
-        </is>
-      </c>
-    </row>
-    <row r="32">
-      <c r="A32" s="2" t="inlineStr">
-        <is>
-          <t>phe_fingertips_92901</t>
-        </is>
-      </c>
-      <c r="B32" s="2" t="inlineStr">
-        <is>
-          <t>Life expectancy inequality at birth by local authority in the South West, 2022 - 24</t>
-        </is>
-      </c>
-      <c r="C32" s="2" t="inlineStr">
-        <is>
-          <t>Fingertips — Inequality in life expectancy at birth (Slope Index of Inequality), Indicator 92901</t>
-        </is>
-      </c>
-      <c r="D32" s="2" t="inlineStr">
-        <is>
-          <t>https://fingertips.phe.org.uk/indicator-details/90/indicator/92901</t>
-        </is>
-      </c>
-      <c r="E32" s="2" t="inlineStr">
-        <is>
-          <t>2022 - 24</t>
-        </is>
-      </c>
-      <c r="F32" s="2" t="inlineStr">
-        <is>
-          <t>three_year_period</t>
-        </is>
-      </c>
-      <c r="G32" s="2" t="n">
-        <v>2022</v>
-      </c>
-      <c r="H32" s="2" t="inlineStr">
-        <is>
-          <t>England</t>
-        </is>
-      </c>
-      <c r="I32" s="2" t="inlineStr">
-        <is>
-          <t>E92000001</t>
-        </is>
-      </c>
-      <c r="J32" s="2" t="inlineStr">
-        <is>
-          <t>England</t>
-        </is>
-      </c>
-      <c r="K32" s="2" t="inlineStr">
-        <is>
-          <t>E92000001</t>
-        </is>
-      </c>
-      <c r="L32" s="2" t="inlineStr">
-        <is>
-          <t>country</t>
-        </is>
-      </c>
-      <c r="M32" s="2" t="inlineStr">
-        <is>
-          <t>life_expectancy_inequality_sii_birth</t>
-        </is>
-      </c>
-      <c r="N32" s="2" t="inlineStr">
-        <is>
-          <t>Slope index of inequality in life expectancy at birth</t>
-        </is>
-      </c>
-      <c r="O32" s="2" t="n">
-        <v>10.373953779621</v>
-      </c>
-      <c r="P32" s="2" t="inlineStr">
-        <is>
-          <t>years</t>
-        </is>
-      </c>
-      <c r="Q32" s="2" t="inlineStr"/>
-      <c r="R32" s="2" t="inlineStr"/>
-      <c r="S32" s="2" t="inlineStr"/>
-      <c r="T32" s="2" t="inlineStr"/>
-      <c r="U32" s="2" t="inlineStr"/>
-      <c r="V32" s="2" t="n">
-        <v>10.2754490660122</v>
-      </c>
-      <c r="W32" s="2" t="n">
-        <v>10.4724763027866</v>
-      </c>
-      <c r="X32" s="2" t="inlineStr"/>
-      <c r="Y32" s="2" t="inlineStr">
-        <is>
-          <t>Male</t>
-        </is>
-      </c>
-      <c r="Z32" s="2" t="inlineStr"/>
-      <c r="AA32" s="2" t="inlineStr"/>
-      <c r="AB32" s="2" t="inlineStr"/>
-      <c r="AC32" s="2" t="inlineStr">
-        <is>
-          <t>{"sex": "Male"}</t>
-        </is>
-      </c>
-      <c r="AD32" s="2" t="inlineStr">
-        <is>
-          <t>Fingertips Indicator 92901</t>
-        </is>
-      </c>
-      <c r="AE32" s="2" t="inlineStr">
-        <is>
-          <t>SII value</t>
-        </is>
-      </c>
-      <c r="AF32" s="2" t="inlineStr"/>
-      <c r="AG32" s="2" t="inlineStr">
-        <is>
-          <t>Direct</t>
-        </is>
-      </c>
-      <c r="AH32" s="2" t="inlineStr"/>
-      <c r="AI32" s="2" t="inlineStr"/>
-      <c r="AJ32" s="2" t="inlineStr">
-        <is>
-          <t>2026-07-22</t>
-        </is>
-      </c>
-    </row>
-    <row r="33">
-      <c r="A33" s="2" t="inlineStr">
-        <is>
-          <t>phe_fingertips_92901</t>
-        </is>
-      </c>
-      <c r="B33" s="2" t="inlineStr">
-        <is>
-          <t>Life expectancy inequality at birth by local authority in the South West, 2022 - 24</t>
-        </is>
-      </c>
-      <c r="C33" s="2" t="inlineStr">
-        <is>
-          <t>Fingertips — Inequality in life expectancy at birth (Slope Index of Inequality), Indicator 92901</t>
-        </is>
-      </c>
-      <c r="D33" s="2" t="inlineStr">
-        <is>
-          <t>https://fingertips.phe.org.uk/indicator-details/90/indicator/92901</t>
-        </is>
-      </c>
-      <c r="E33" s="2" t="inlineStr">
-        <is>
-          <t>2022 - 24</t>
-        </is>
-      </c>
-      <c r="F33" s="2" t="inlineStr">
-        <is>
-          <t>three_year_period</t>
-        </is>
-      </c>
-      <c r="G33" s="2" t="n">
-        <v>2022</v>
-      </c>
-      <c r="H33" s="2" t="inlineStr">
-        <is>
-          <t>England</t>
-        </is>
-      </c>
-      <c r="I33" s="2" t="inlineStr">
-        <is>
-          <t>E92000001</t>
-        </is>
-      </c>
-      <c r="J33" s="2" t="inlineStr">
-        <is>
-          <t>England</t>
-        </is>
-      </c>
-      <c r="K33" s="2" t="inlineStr">
-        <is>
-          <t>E92000001</t>
-        </is>
-      </c>
-      <c r="L33" s="2" t="inlineStr">
-        <is>
-          <t>country</t>
-        </is>
-      </c>
-      <c r="M33" s="2" t="inlineStr">
-        <is>
-          <t>life_expectancy_inequality_sii_birth</t>
-        </is>
-      </c>
-      <c r="N33" s="2" t="inlineStr">
-        <is>
-          <t>Slope index of inequality in life expectancy at birth</t>
-        </is>
-      </c>
-      <c r="O33" s="2" t="n">
-        <v>74.1627665862413</v>
-      </c>
-      <c r="P33" s="2" t="inlineStr">
-        <is>
-          <t>years</t>
-        </is>
-      </c>
-      <c r="Q33" s="2" t="inlineStr"/>
-      <c r="R33" s="2" t="inlineStr"/>
-      <c r="S33" s="2" t="inlineStr"/>
-      <c r="T33" s="2" t="inlineStr"/>
-      <c r="U33" s="2" t="inlineStr"/>
-      <c r="V33" s="2" t="n"/>
-      <c r="W33" s="2" t="n"/>
-      <c r="X33" s="2" t="inlineStr"/>
-      <c r="Y33" s="2" t="inlineStr">
-        <is>
-          <t>Male</t>
-        </is>
-      </c>
-      <c r="Z33" s="2" t="inlineStr"/>
-      <c r="AA33" s="2" t="inlineStr"/>
-      <c r="AB33" s="2" t="inlineStr"/>
-      <c r="AC33" s="2" t="inlineStr">
-        <is>
-          <t>{"sex": "Male"}</t>
-        </is>
-      </c>
-      <c r="AD33" s="2" t="inlineStr">
-        <is>
-          <t>Fingertips Indicator 92901</t>
-        </is>
-      </c>
-      <c r="AE33" s="2" t="inlineStr">
-        <is>
-          <t>Limits for SII regression charts</t>
-        </is>
-      </c>
-      <c r="AF33" s="2" t="inlineStr"/>
-      <c r="AG33" s="2" t="inlineStr">
-        <is>
-          <t>Direct</t>
-        </is>
-      </c>
-      <c r="AH33" s="2" t="inlineStr"/>
-      <c r="AI33" s="2" t="inlineStr"/>
-      <c r="AJ33" s="2" t="inlineStr">
-        <is>
-          <t>2026-07-22</t>
-        </is>
-      </c>
-    </row>
-    <row r="34">
-      <c r="A34" s="2" t="inlineStr">
-        <is>
-          <t>phe_fingertips_92901</t>
-        </is>
-      </c>
-      <c r="B34" s="2" t="inlineStr">
-        <is>
-          <t>Life expectancy inequality at birth by local authority in the South West, 2022 - 24</t>
-        </is>
-      </c>
-      <c r="C34" s="2" t="inlineStr">
-        <is>
-          <t>Fingertips — Inequality in life expectancy at birth (Slope Index of Inequality), Indicator 92901</t>
-        </is>
-      </c>
-      <c r="D34" s="2" t="inlineStr">
-        <is>
-          <t>https://fingertips.phe.org.uk/indicator-details/90/indicator/92901</t>
-        </is>
-      </c>
-      <c r="E34" s="2" t="inlineStr">
-        <is>
-          <t>2022 - 24</t>
-        </is>
-      </c>
-      <c r="F34" s="2" t="inlineStr">
-        <is>
-          <t>three_year_period</t>
-        </is>
-      </c>
-      <c r="G34" s="2" t="n">
-        <v>2022</v>
-      </c>
-      <c r="H34" s="2" t="inlineStr">
-        <is>
-          <t>South West region (statistical)</t>
-        </is>
-      </c>
-      <c r="I34" s="2" t="inlineStr">
-        <is>
-          <t>E12000009</t>
-        </is>
-      </c>
-      <c r="J34" s="2" t="inlineStr">
-        <is>
-          <t>South West region (statistical)</t>
-        </is>
-      </c>
-      <c r="K34" s="2" t="inlineStr">
-        <is>
-          <t>E12000009</t>
-        </is>
-      </c>
-      <c r="L34" s="2" t="inlineStr">
-        <is>
-          <t>region</t>
-        </is>
-      </c>
-      <c r="M34" s="2" t="inlineStr">
-        <is>
-          <t>life_expectancy_inequality_sii_birth</t>
-        </is>
-      </c>
-      <c r="N34" s="2" t="inlineStr">
-        <is>
-          <t>Slope index of inequality in life expectancy at birth</t>
-        </is>
-      </c>
-      <c r="O34" s="2" t="n">
-        <v>5.59964175909663</v>
-      </c>
-      <c r="P34" s="2" t="inlineStr">
-        <is>
-          <t>years</t>
-        </is>
-      </c>
-      <c r="Q34" s="2" t="inlineStr"/>
-      <c r="R34" s="2" t="inlineStr"/>
-      <c r="S34" s="2" t="inlineStr"/>
-      <c r="T34" s="2" t="inlineStr"/>
-      <c r="U34" s="2" t="inlineStr"/>
-      <c r="V34" s="2" t="n">
-        <v>5.31888872864678</v>
-      </c>
-      <c r="W34" s="2" t="n">
-        <v>5.88052225585969</v>
-      </c>
-      <c r="X34" s="2" t="inlineStr"/>
-      <c r="Y34" s="2" t="inlineStr">
-        <is>
-          <t>Female</t>
-        </is>
-      </c>
-      <c r="Z34" s="2" t="inlineStr"/>
-      <c r="AA34" s="2" t="inlineStr"/>
-      <c r="AB34" s="2" t="inlineStr"/>
-      <c r="AC34" s="2" t="inlineStr">
-        <is>
-          <t>{"sex": "Female"}</t>
-        </is>
-      </c>
-      <c r="AD34" s="2" t="inlineStr">
-        <is>
-          <t>Fingertips Indicator 92901</t>
-        </is>
-      </c>
-      <c r="AE34" s="2" t="inlineStr">
-        <is>
-          <t>SII value</t>
-        </is>
-      </c>
-      <c r="AF34" s="2" t="inlineStr"/>
-      <c r="AG34" s="2" t="inlineStr">
-        <is>
-          <t>Direct</t>
-        </is>
-      </c>
-      <c r="AH34" s="2" t="inlineStr"/>
-      <c r="AI34" s="2" t="inlineStr"/>
-      <c r="AJ34" s="2" t="inlineStr">
-        <is>
-          <t>2026-07-22</t>
-        </is>
-      </c>
-    </row>
-    <row r="35">
-      <c r="A35" s="2" t="inlineStr">
-        <is>
-          <t>phe_fingertips_92901</t>
-        </is>
-      </c>
-      <c r="B35" s="2" t="inlineStr">
-        <is>
-          <t>Life expectancy inequality at birth by local authority in the South West, 2022 - 24</t>
-        </is>
-      </c>
-      <c r="C35" s="2" t="inlineStr">
-        <is>
-          <t>Fingertips — Inequality in life expectancy at birth (Slope Index of Inequality), Indicator 92901</t>
-        </is>
-      </c>
-      <c r="D35" s="2" t="inlineStr">
-        <is>
-          <t>https://fingertips.phe.org.uk/indicator-details/90/indicator/92901</t>
-        </is>
-      </c>
-      <c r="E35" s="2" t="inlineStr">
-        <is>
-          <t>2022 - 24</t>
-        </is>
-      </c>
-      <c r="F35" s="2" t="inlineStr">
-        <is>
-          <t>three_year_period</t>
-        </is>
-      </c>
-      <c r="G35" s="2" t="n">
-        <v>2022</v>
-      </c>
-      <c r="H35" s="2" t="inlineStr">
-        <is>
-          <t>South West region (statistical)</t>
-        </is>
-      </c>
-      <c r="I35" s="2" t="inlineStr">
-        <is>
-          <t>E12000009</t>
-        </is>
-      </c>
-      <c r="J35" s="2" t="inlineStr">
-        <is>
-          <t>South West region (statistical)</t>
-        </is>
-      </c>
-      <c r="K35" s="2" t="inlineStr">
-        <is>
-          <t>E12000009</t>
-        </is>
-      </c>
-      <c r="L35" s="2" t="inlineStr">
-        <is>
-          <t>region</t>
-        </is>
-      </c>
-      <c r="M35" s="2" t="inlineStr">
-        <is>
-          <t>life_expectancy_inequality_sii_birth</t>
-        </is>
-      </c>
-      <c r="N35" s="2" t="inlineStr">
-        <is>
-          <t>Slope index of inequality in life expectancy at birth</t>
-        </is>
-      </c>
-      <c r="O35" s="2" t="n">
-        <v>81.2876019454278</v>
-      </c>
-      <c r="P35" s="2" t="inlineStr">
-        <is>
-          <t>years</t>
-        </is>
-      </c>
-      <c r="Q35" s="2" t="inlineStr"/>
-      <c r="R35" s="2" t="inlineStr"/>
-      <c r="S35" s="2" t="inlineStr"/>
-      <c r="T35" s="2" t="inlineStr"/>
-      <c r="U35" s="2" t="inlineStr"/>
-      <c r="V35" s="2" t="n"/>
-      <c r="W35" s="2" t="n"/>
-      <c r="X35" s="2" t="inlineStr"/>
-      <c r="Y35" s="2" t="inlineStr">
-        <is>
-          <t>Female</t>
-        </is>
-      </c>
-      <c r="Z35" s="2" t="inlineStr"/>
-      <c r="AA35" s="2" t="inlineStr"/>
-      <c r="AB35" s="2" t="inlineStr"/>
-      <c r="AC35" s="2" t="inlineStr">
-        <is>
-          <t>{"sex": "Female"}</t>
-        </is>
-      </c>
-      <c r="AD35" s="2" t="inlineStr">
-        <is>
-          <t>Fingertips Indicator 92901</t>
-        </is>
-      </c>
-      <c r="AE35" s="2" t="inlineStr">
-        <is>
-          <t>Limits for SII regression charts</t>
-        </is>
-      </c>
-      <c r="AF35" s="2" t="inlineStr"/>
-      <c r="AG35" s="2" t="inlineStr">
-        <is>
-          <t>Direct</t>
-        </is>
-      </c>
-      <c r="AH35" s="2" t="inlineStr"/>
-      <c r="AI35" s="2" t="inlineStr"/>
-      <c r="AJ35" s="2" t="inlineStr">
-        <is>
-          <t>2026-07-22</t>
-        </is>
-      </c>
-    </row>
-    <row r="36">
-      <c r="A36" s="2" t="inlineStr">
-        <is>
-          <t>phe_fingertips_92901</t>
-        </is>
-      </c>
-      <c r="B36" s="2" t="inlineStr">
-        <is>
-          <t>Life expectancy inequality at birth by local authority in the South West, 2022 - 24</t>
-        </is>
-      </c>
-      <c r="C36" s="2" t="inlineStr">
-        <is>
-          <t>Fingertips — Inequality in life expectancy at birth (Slope Index of Inequality), Indicator 92901</t>
-        </is>
-      </c>
-      <c r="D36" s="2" t="inlineStr">
-        <is>
-          <t>https://fingertips.phe.org.uk/indicator-details/90/indicator/92901</t>
-        </is>
-      </c>
-      <c r="E36" s="2" t="inlineStr">
-        <is>
-          <t>2022 - 24</t>
-        </is>
-      </c>
-      <c r="F36" s="2" t="inlineStr">
-        <is>
-          <t>three_year_period</t>
-        </is>
-      </c>
-      <c r="G36" s="2" t="n">
-        <v>2022</v>
-      </c>
-      <c r="H36" s="2" t="inlineStr">
-        <is>
-          <t>South West region (statistical)</t>
-        </is>
-      </c>
-      <c r="I36" s="2" t="inlineStr">
-        <is>
-          <t>E12000009</t>
-        </is>
-      </c>
-      <c r="J36" s="2" t="inlineStr">
-        <is>
-          <t>South West region (statistical)</t>
-        </is>
-      </c>
-      <c r="K36" s="2" t="inlineStr">
-        <is>
-          <t>E12000009</t>
-        </is>
-      </c>
-      <c r="L36" s="2" t="inlineStr">
-        <is>
-          <t>region</t>
-        </is>
-      </c>
-      <c r="M36" s="2" t="inlineStr">
-        <is>
-          <t>life_expectancy_inequality_sii_birth</t>
-        </is>
-      </c>
-      <c r="N36" s="2" t="inlineStr">
-        <is>
-          <t>Slope index of inequality in life expectancy at birth</t>
-        </is>
-      </c>
-      <c r="O36" s="2" t="n">
-        <v>7.78126329187077</v>
-      </c>
-      <c r="P36" s="2" t="inlineStr">
-        <is>
-          <t>years</t>
-        </is>
-      </c>
-      <c r="Q36" s="2" t="inlineStr"/>
-      <c r="R36" s="2" t="inlineStr"/>
-      <c r="S36" s="2" t="inlineStr"/>
-      <c r="T36" s="2" t="inlineStr"/>
-      <c r="U36" s="2" t="inlineStr"/>
-      <c r="V36" s="2" t="n">
-        <v>7.4785922356622</v>
-      </c>
-      <c r="W36" s="2" t="n">
-        <v>8.08262609624769</v>
-      </c>
-      <c r="X36" s="2" t="inlineStr"/>
-      <c r="Y36" s="2" t="inlineStr">
-        <is>
-          <t>Male</t>
-        </is>
-      </c>
-      <c r="Z36" s="2" t="inlineStr"/>
-      <c r="AA36" s="2" t="inlineStr"/>
-      <c r="AB36" s="2" t="inlineStr"/>
-      <c r="AC36" s="2" t="inlineStr">
-        <is>
-          <t>{"sex": "Male"}</t>
-        </is>
-      </c>
-      <c r="AD36" s="2" t="inlineStr">
-        <is>
-          <t>Fingertips Indicator 92901</t>
-        </is>
-      </c>
-      <c r="AE36" s="2" t="inlineStr">
-        <is>
-          <t>SII value</t>
-        </is>
-      </c>
-      <c r="AF36" s="2" t="inlineStr"/>
-      <c r="AG36" s="2" t="inlineStr">
-        <is>
-          <t>Direct</t>
-        </is>
-      </c>
-      <c r="AH36" s="2" t="inlineStr"/>
-      <c r="AI36" s="2" t="inlineStr"/>
-      <c r="AJ36" s="2" t="inlineStr">
-        <is>
-          <t>2026-07-22</t>
-        </is>
-      </c>
-    </row>
-    <row r="37">
-      <c r="A37" s="2" t="inlineStr">
-        <is>
-          <t>phe_fingertips_92901</t>
-        </is>
-      </c>
-      <c r="B37" s="2" t="inlineStr">
-        <is>
-          <t>Life expectancy inequality at birth by local authority in the South West, 2022 - 24</t>
-        </is>
-      </c>
-      <c r="C37" s="2" t="inlineStr">
-        <is>
-          <t>Fingertips — Inequality in life expectancy at birth (Slope Index of Inequality), Indicator 92901</t>
-        </is>
-      </c>
-      <c r="D37" s="2" t="inlineStr">
-        <is>
-          <t>https://fingertips.phe.org.uk/indicator-details/90/indicator/92901</t>
-        </is>
-      </c>
-      <c r="E37" s="2" t="inlineStr">
-        <is>
-          <t>2022 - 24</t>
-        </is>
-      </c>
-      <c r="F37" s="2" t="inlineStr">
-        <is>
-          <t>three_year_period</t>
-        </is>
-      </c>
-      <c r="G37" s="2" t="n">
-        <v>2022</v>
-      </c>
-      <c r="H37" s="2" t="inlineStr">
-        <is>
-          <t>South West region (statistical)</t>
-        </is>
-      </c>
-      <c r="I37" s="2" t="inlineStr">
-        <is>
-          <t>E12000009</t>
-        </is>
-      </c>
-      <c r="J37" s="2" t="inlineStr">
-        <is>
-          <t>South West region (statistical)</t>
-        </is>
-      </c>
-      <c r="K37" s="2" t="inlineStr">
-        <is>
-          <t>E12000009</t>
-        </is>
-      </c>
-      <c r="L37" s="2" t="inlineStr">
-        <is>
-          <t>region</t>
-        </is>
-      </c>
-      <c r="M37" s="2" t="inlineStr">
-        <is>
-          <t>life_expectancy_inequality_sii_birth</t>
-        </is>
-      </c>
-      <c r="N37" s="2" t="inlineStr">
-        <is>
-          <t>Slope index of inequality in life expectancy at birth</t>
-        </is>
-      </c>
-      <c r="O37" s="2" t="n">
-        <v>76.38941705519851</v>
-      </c>
-      <c r="P37" s="2" t="inlineStr">
-        <is>
-          <t>years</t>
-        </is>
-      </c>
-      <c r="Q37" s="2" t="inlineStr"/>
-      <c r="R37" s="2" t="inlineStr"/>
-      <c r="S37" s="2" t="inlineStr"/>
-      <c r="T37" s="2" t="inlineStr"/>
-      <c r="U37" s="2" t="inlineStr"/>
-      <c r="V37" s="2" t="n"/>
-      <c r="W37" s="2" t="n"/>
-      <c r="X37" s="2" t="inlineStr"/>
-      <c r="Y37" s="2" t="inlineStr">
-        <is>
-          <t>Male</t>
-        </is>
-      </c>
-      <c r="Z37" s="2" t="inlineStr"/>
-      <c r="AA37" s="2" t="inlineStr"/>
-      <c r="AB37" s="2" t="inlineStr"/>
-      <c r="AC37" s="2" t="inlineStr">
-        <is>
-          <t>{"sex": "Male"}</t>
-        </is>
-      </c>
-      <c r="AD37" s="2" t="inlineStr">
-        <is>
-          <t>Fingertips Indicator 92901</t>
-        </is>
-      </c>
-      <c r="AE37" s="2" t="inlineStr">
-        <is>
-          <t>Limits for SII regression charts</t>
-        </is>
-      </c>
-      <c r="AF37" s="2" t="inlineStr"/>
-      <c r="AG37" s="2" t="inlineStr">
-        <is>
-          <t>Direct</t>
-        </is>
-      </c>
-      <c r="AH37" s="2" t="inlineStr"/>
-      <c r="AI37" s="2" t="inlineStr"/>
-      <c r="AJ37" s="2" t="inlineStr">
-        <is>
-          <t>2026-07-22</t>
-        </is>
-      </c>
-    </row>
-    <row r="38">
-      <c r="A38" s="2" t="inlineStr">
-        <is>
-          <t>phe_fingertips_92901</t>
-        </is>
-      </c>
-      <c r="B38" s="2" t="inlineStr">
-        <is>
-          <t>Life expectancy inequality at birth by local authority in the South West, 2022 - 24</t>
-        </is>
-      </c>
-      <c r="C38" s="2" t="inlineStr">
-        <is>
-          <t>Fingertips — Inequality in life expectancy at birth (Slope Index of Inequality), Indicator 92901</t>
-        </is>
-      </c>
-      <c r="D38" s="2" t="inlineStr">
-        <is>
-          <t>https://fingertips.phe.org.uk/indicator-details/90/indicator/92901</t>
-        </is>
-      </c>
-      <c r="E38" s="2" t="inlineStr">
-        <is>
-          <t>2022 - 24</t>
-        </is>
-      </c>
-      <c r="F38" s="2" t="inlineStr">
-        <is>
-          <t>three_year_period</t>
-        </is>
-      </c>
-      <c r="G38" s="2" t="n">
-        <v>2022</v>
-      </c>
-      <c r="H38" s="2" t="inlineStr">
-        <is>
-          <t>London region (statistical)</t>
-        </is>
-      </c>
-      <c r="I38" s="2" t="inlineStr">
-        <is>
-          <t>E12000007</t>
-        </is>
-      </c>
-      <c r="J38" s="2" t="inlineStr">
-        <is>
-          <t>London region (statistical)</t>
-        </is>
-      </c>
-      <c r="K38" s="2" t="inlineStr">
-        <is>
-          <t>E12000007</t>
-        </is>
-      </c>
-      <c r="L38" s="2" t="inlineStr">
-        <is>
-          <t>region</t>
-        </is>
-      </c>
-      <c r="M38" s="2" t="inlineStr">
-        <is>
-          <t>life_expectancy_inequality_sii_birth</t>
-        </is>
-      </c>
-      <c r="N38" s="2" t="inlineStr">
-        <is>
-          <t>Slope index of inequality in life expectancy at birth</t>
-        </is>
-      </c>
-      <c r="O38" s="2" t="n">
-        <v>4.74617067288794</v>
-      </c>
-      <c r="P38" s="2" t="inlineStr">
-        <is>
-          <t>years</t>
-        </is>
-      </c>
-      <c r="Q38" s="2" t="inlineStr"/>
-      <c r="R38" s="2" t="inlineStr"/>
-      <c r="S38" s="2" t="inlineStr"/>
-      <c r="T38" s="2" t="inlineStr"/>
-      <c r="U38" s="2" t="inlineStr"/>
-      <c r="V38" s="2" t="n">
-        <v>4.4817708429787</v>
-      </c>
-      <c r="W38" s="2" t="n">
-        <v>5.00970035756127</v>
-      </c>
-      <c r="X38" s="2" t="inlineStr"/>
-      <c r="Y38" s="2" t="inlineStr">
-        <is>
-          <t>Female</t>
-        </is>
-      </c>
-      <c r="Z38" s="2" t="inlineStr"/>
-      <c r="AA38" s="2" t="inlineStr"/>
-      <c r="AB38" s="2" t="inlineStr"/>
-      <c r="AC38" s="2" t="inlineStr">
-        <is>
-          <t>{"sex": "Female"}</t>
-        </is>
-      </c>
-      <c r="AD38" s="2" t="inlineStr">
-        <is>
-          <t>Fingertips Indicator 92901</t>
-        </is>
-      </c>
-      <c r="AE38" s="2" t="inlineStr">
-        <is>
-          <t>SII value</t>
-        </is>
-      </c>
-      <c r="AF38" s="2" t="inlineStr"/>
-      <c r="AG38" s="2" t="inlineStr">
-        <is>
-          <t>Direct</t>
-        </is>
-      </c>
-      <c r="AH38" s="2" t="inlineStr"/>
-      <c r="AI38" s="2" t="inlineStr"/>
-      <c r="AJ38" s="2" t="inlineStr">
-        <is>
-          <t>2026-07-22</t>
-        </is>
-      </c>
-    </row>
-    <row r="39">
-      <c r="A39" s="2" t="inlineStr">
-        <is>
-          <t>phe_fingertips_92901</t>
-        </is>
-      </c>
-      <c r="B39" s="2" t="inlineStr">
-        <is>
-          <t>Life expectancy inequality at birth by local authority in the South West, 2022 - 24</t>
-        </is>
-      </c>
-      <c r="C39" s="2" t="inlineStr">
-        <is>
-          <t>Fingertips — Inequality in life expectancy at birth (Slope Index of Inequality), Indicator 92901</t>
-        </is>
-      </c>
-      <c r="D39" s="2" t="inlineStr">
-        <is>
-          <t>https://fingertips.phe.org.uk/indicator-details/90/indicator/92901</t>
-        </is>
-      </c>
-      <c r="E39" s="2" t="inlineStr">
-        <is>
-          <t>2022 - 24</t>
-        </is>
-      </c>
-      <c r="F39" s="2" t="inlineStr">
-        <is>
-          <t>three_year_period</t>
-        </is>
-      </c>
-      <c r="G39" s="2" t="n">
-        <v>2022</v>
-      </c>
-      <c r="H39" s="2" t="inlineStr">
-        <is>
-          <t>London region (statistical)</t>
-        </is>
-      </c>
-      <c r="I39" s="2" t="inlineStr">
-        <is>
-          <t>E12000007</t>
-        </is>
-      </c>
-      <c r="J39" s="2" t="inlineStr">
-        <is>
-          <t>London region (statistical)</t>
-        </is>
-      </c>
-      <c r="K39" s="2" t="inlineStr">
-        <is>
-          <t>E12000007</t>
-        </is>
-      </c>
-      <c r="L39" s="2" t="inlineStr">
-        <is>
-          <t>region</t>
-        </is>
-      </c>
-      <c r="M39" s="2" t="inlineStr">
-        <is>
-          <t>life_expectancy_inequality_sii_birth</t>
-        </is>
-      </c>
-      <c r="N39" s="2" t="inlineStr">
-        <is>
-          <t>Slope index of inequality in life expectancy at birth</t>
-        </is>
-      </c>
-      <c r="O39" s="2" t="n">
-        <v>82.15862008585481</v>
-      </c>
-      <c r="P39" s="2" t="inlineStr">
-        <is>
-          <t>years</t>
-        </is>
-      </c>
-      <c r="Q39" s="2" t="inlineStr"/>
-      <c r="R39" s="2" t="inlineStr"/>
-      <c r="S39" s="2" t="inlineStr"/>
-      <c r="T39" s="2" t="inlineStr"/>
-      <c r="U39" s="2" t="inlineStr"/>
-      <c r="V39" s="2" t="n"/>
-      <c r="W39" s="2" t="n"/>
-      <c r="X39" s="2" t="inlineStr"/>
-      <c r="Y39" s="2" t="inlineStr">
-        <is>
-          <t>Female</t>
-        </is>
-      </c>
-      <c r="Z39" s="2" t="inlineStr"/>
-      <c r="AA39" s="2" t="inlineStr"/>
-      <c r="AB39" s="2" t="inlineStr"/>
-      <c r="AC39" s="2" t="inlineStr">
-        <is>
-          <t>{"sex": "Female"}</t>
-        </is>
-      </c>
-      <c r="AD39" s="2" t="inlineStr">
-        <is>
-          <t>Fingertips Indicator 92901</t>
-        </is>
-      </c>
-      <c r="AE39" s="2" t="inlineStr">
-        <is>
-          <t>Limits for SII regression charts</t>
-        </is>
-      </c>
-      <c r="AF39" s="2" t="inlineStr"/>
-      <c r="AG39" s="2" t="inlineStr">
-        <is>
-          <t>Direct</t>
-        </is>
-      </c>
-      <c r="AH39" s="2" t="inlineStr"/>
-      <c r="AI39" s="2" t="inlineStr"/>
-      <c r="AJ39" s="2" t="inlineStr">
-        <is>
-          <t>2026-07-22</t>
-        </is>
-      </c>
-    </row>
-    <row r="40">
-      <c r="A40" s="2" t="inlineStr">
-        <is>
-          <t>phe_fingertips_92901</t>
-        </is>
-      </c>
-      <c r="B40" s="2" t="inlineStr">
-        <is>
-          <t>Life expectancy inequality at birth by local authority in the South West, 2022 - 24</t>
-        </is>
-      </c>
-      <c r="C40" s="2" t="inlineStr">
-        <is>
-          <t>Fingertips — Inequality in life expectancy at birth (Slope Index of Inequality), Indicator 92901</t>
-        </is>
-      </c>
-      <c r="D40" s="2" t="inlineStr">
-        <is>
-          <t>https://fingertips.phe.org.uk/indicator-details/90/indicator/92901</t>
-        </is>
-      </c>
-      <c r="E40" s="2" t="inlineStr">
-        <is>
-          <t>2022 - 24</t>
-        </is>
-      </c>
-      <c r="F40" s="2" t="inlineStr">
-        <is>
-          <t>three_year_period</t>
-        </is>
-      </c>
-      <c r="G40" s="2" t="n">
-        <v>2022</v>
-      </c>
-      <c r="H40" s="2" t="inlineStr">
-        <is>
-          <t>London region (statistical)</t>
-        </is>
-      </c>
-      <c r="I40" s="2" t="inlineStr">
-        <is>
-          <t>E12000007</t>
-        </is>
-      </c>
-      <c r="J40" s="2" t="inlineStr">
-        <is>
-          <t>London region (statistical)</t>
-        </is>
-      </c>
-      <c r="K40" s="2" t="inlineStr">
-        <is>
-          <t>E12000007</t>
-        </is>
-      </c>
-      <c r="L40" s="2" t="inlineStr">
-        <is>
-          <t>region</t>
-        </is>
-      </c>
-      <c r="M40" s="2" t="inlineStr">
-        <is>
-          <t>life_expectancy_inequality_sii_birth</t>
-        </is>
-      </c>
-      <c r="N40" s="2" t="inlineStr">
-        <is>
-          <t>Slope index of inequality in life expectancy at birth</t>
-        </is>
-      </c>
-      <c r="O40" s="2" t="n">
-        <v>7.85755327065507</v>
-      </c>
-      <c r="P40" s="2" t="inlineStr">
-        <is>
-          <t>years</t>
-        </is>
-      </c>
-      <c r="Q40" s="2" t="inlineStr"/>
-      <c r="R40" s="2" t="inlineStr"/>
-      <c r="S40" s="2" t="inlineStr"/>
-      <c r="T40" s="2" t="inlineStr"/>
-      <c r="U40" s="2" t="inlineStr"/>
-      <c r="V40" s="2" t="n">
-        <v>7.58923901627381</v>
-      </c>
-      <c r="W40" s="2" t="n">
-        <v>8.125845973842219</v>
-      </c>
-      <c r="X40" s="2" t="inlineStr"/>
-      <c r="Y40" s="2" t="inlineStr">
-        <is>
-          <t>Male</t>
-        </is>
-      </c>
-      <c r="Z40" s="2" t="inlineStr"/>
-      <c r="AA40" s="2" t="inlineStr"/>
-      <c r="AB40" s="2" t="inlineStr"/>
-      <c r="AC40" s="2" t="inlineStr">
-        <is>
-          <t>{"sex": "Male"}</t>
-        </is>
-      </c>
-      <c r="AD40" s="2" t="inlineStr">
-        <is>
-          <t>Fingertips Indicator 92901</t>
-        </is>
-      </c>
-      <c r="AE40" s="2" t="inlineStr">
-        <is>
-          <t>SII value</t>
-        </is>
-      </c>
-      <c r="AF40" s="2" t="inlineStr"/>
-      <c r="AG40" s="2" t="inlineStr">
-        <is>
-          <t>Direct</t>
-        </is>
-      </c>
-      <c r="AH40" s="2" t="inlineStr"/>
-      <c r="AI40" s="2" t="inlineStr"/>
-      <c r="AJ40" s="2" t="inlineStr">
-        <is>
-          <t>2026-07-22</t>
-        </is>
-      </c>
-    </row>
-    <row r="41">
-      <c r="A41" s="2" t="inlineStr">
-        <is>
-          <t>phe_fingertips_92901</t>
-        </is>
-      </c>
-      <c r="B41" s="2" t="inlineStr">
-        <is>
-          <t>Life expectancy inequality at birth by local authority in the South West, 2022 - 24</t>
-        </is>
-      </c>
-      <c r="C41" s="2" t="inlineStr">
-        <is>
-          <t>Fingertips — Inequality in life expectancy at birth (Slope Index of Inequality), Indicator 92901</t>
-        </is>
-      </c>
-      <c r="D41" s="2" t="inlineStr">
-        <is>
-          <t>https://fingertips.phe.org.uk/indicator-details/90/indicator/92901</t>
-        </is>
-      </c>
-      <c r="E41" s="2" t="inlineStr">
-        <is>
-          <t>2022 - 24</t>
-        </is>
-      </c>
-      <c r="F41" s="2" t="inlineStr">
-        <is>
-          <t>three_year_period</t>
-        </is>
-      </c>
-      <c r="G41" s="2" t="n">
-        <v>2022</v>
-      </c>
-      <c r="H41" s="2" t="inlineStr">
-        <is>
-          <t>London region (statistical)</t>
-        </is>
-      </c>
-      <c r="I41" s="2" t="inlineStr">
-        <is>
-          <t>E12000007</t>
-        </is>
-      </c>
-      <c r="J41" s="2" t="inlineStr">
-        <is>
-          <t>London region (statistical)</t>
-        </is>
-      </c>
-      <c r="K41" s="2" t="inlineStr">
-        <is>
-          <t>E12000007</t>
-        </is>
-      </c>
-      <c r="L41" s="2" t="inlineStr">
-        <is>
-          <t>region</t>
-        </is>
-      </c>
-      <c r="M41" s="2" t="inlineStr">
-        <is>
-          <t>life_expectancy_inequality_sii_birth</t>
-        </is>
-      </c>
-      <c r="N41" s="2" t="inlineStr">
-        <is>
-          <t>Slope index of inequality in life expectancy at birth</t>
-        </is>
-      </c>
-      <c r="O41" s="2" t="n">
-        <v>76.33508478900821</v>
-      </c>
-      <c r="P41" s="2" t="inlineStr">
-        <is>
-          <t>years</t>
-        </is>
-      </c>
-      <c r="Q41" s="2" t="inlineStr"/>
-      <c r="R41" s="2" t="inlineStr"/>
-      <c r="S41" s="2" t="inlineStr"/>
-      <c r="T41" s="2" t="inlineStr"/>
-      <c r="U41" s="2" t="inlineStr"/>
-      <c r="V41" s="2" t="n"/>
-      <c r="W41" s="2" t="n"/>
-      <c r="X41" s="2" t="inlineStr"/>
-      <c r="Y41" s="2" t="inlineStr">
-        <is>
-          <t>Male</t>
-        </is>
-      </c>
-      <c r="Z41" s="2" t="inlineStr"/>
-      <c r="AA41" s="2" t="inlineStr"/>
-      <c r="AB41" s="2" t="inlineStr"/>
-      <c r="AC41" s="2" t="inlineStr">
-        <is>
-          <t>{"sex": "Male"}</t>
-        </is>
-      </c>
-      <c r="AD41" s="2" t="inlineStr">
-        <is>
-          <t>Fingertips Indicator 92901</t>
-        </is>
-      </c>
-      <c r="AE41" s="2" t="inlineStr">
-        <is>
-          <t>Limits for SII regression charts</t>
-        </is>
-      </c>
-      <c r="AF41" s="2" t="inlineStr"/>
-      <c r="AG41" s="2" t="inlineStr">
-        <is>
-          <t>Direct</t>
-        </is>
-      </c>
-      <c r="AH41" s="2" t="inlineStr"/>
-      <c r="AI41" s="2" t="inlineStr"/>
-      <c r="AJ41" s="2" t="inlineStr">
         <is>
           <t>2026-07-22</t>
         </is>

</xml_diff>